<commit_message>
Refactor codebase: add .gitignore, standardize Python code, clean workflow & update README
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-14T22:45</t>
+          <t>2026-09-14T23:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,16 +539,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25.3</v>
+        <v>25.1</v>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>7.1</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Include visualization generation in daily workflow
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-14T23:00</t>
+          <t>2026-09-14T23:15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25.1</v>
+        <v>25</v>
       </c>
       <c r="E4" t="n">
         <v>81</v>
@@ -548,7 +548,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Add full Telangana 33 districts reporting and statewide analytics dashboard
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="District_Daily_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Telangana_State_Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +425,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>state</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -455,71 +456,86 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>weather_code</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>observation_time</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-12T09:00</t>
+          <t>Adilabad</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29.4</v>
+        <v>25.1</v>
       </c>
       <c r="E2" t="n">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-13T09:00</t>
+          <t>Bhadradri Kothagudem</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>28.1</v>
+        <v>25</v>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="F3" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>9.800000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="H3" t="n">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -530,28 +546,1285 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-14T23:15</t>
+          <t>Hanumakonda</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="E4" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>82</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>92</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>94</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E10" t="n">
+        <v>89</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" t="n">
+        <v>82</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>93</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>93</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E14" t="n">
+        <v>95</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>79</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="E16" t="n">
+        <v>87</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>85</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="E18" t="n">
+        <v>84</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" t="n">
+        <v>96</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>86</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>88</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" t="n">
+        <v>75</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>85</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E24" t="n">
+        <v>79</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>87</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>83</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>82</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>79</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>82</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>94</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="E31" t="n">
+        <v>81</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>69</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>94</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>86</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>9</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-09-14T23:45</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_districts_monitored</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>state_avg_temp_C</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hottest_district</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>max_temp_C</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>coolest_district</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>min_temp_C</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>state_avg_humidity_%</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>total_state_rainfall_mm</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>rainiest_district</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>max_rainfall_mm</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>windiest_district</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>max_wind_speed_kmh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I2" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>12.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add SQLite DB storage, monthly reports, and daily/monthly picture archives
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="District_Daily_Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Telangana_State_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly_Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1812,7 +1813,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Bhadradri Kothagudem</t>
+          <t>Jangaon</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -1825,6 +1826,948 @@
       </c>
       <c r="N2" t="n">
         <v>12.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>monthly_avg_temp_C</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>monthly_max_temp_C</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>monthly_min_temp_C</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>monthly_avg_humidity_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>monthly_total_rain_mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>87</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>96</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F4" t="n">
+        <v>94</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>82</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>80</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>92</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>94</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E10" t="n">
+        <v>23</v>
+      </c>
+      <c r="F10" t="n">
+        <v>89</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" t="n">
+        <v>26</v>
+      </c>
+      <c r="F11" t="n">
+        <v>82</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>93</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>93</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D14" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E14" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>95</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>79</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="D16" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="E16" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>87</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>85</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="E18" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>84</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>24</v>
+      </c>
+      <c r="D19" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" t="n">
+        <v>96</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D20" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F20" t="n">
+        <v>86</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>88</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" t="n">
+        <v>25</v>
+      </c>
+      <c r="F22" t="n">
+        <v>75</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D23" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>85</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D24" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E24" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F24" t="n">
+        <v>79</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D25" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F25" t="n">
+        <v>87</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>83</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>82</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D28" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>79</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>82</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="F30" t="n">
+        <v>94</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="D31" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="E31" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="F31" t="n">
+        <v>81</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="F32" t="n">
+        <v>69</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D33" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>94</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D34" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>86</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest weather data files
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2887,23 +2887,23 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>32.5</v>
+        <v>28.7</v>
       </c>
       <c r="E67" t="n">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="F67" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>4.7</v>
+        <v>1.4</v>
       </c>
       <c r="H67" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -2924,23 +2924,23 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>32.6</v>
+        <v>29.7</v>
       </c>
       <c r="E68" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>4.4</v>
+        <v>7.6</v>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -2961,23 +2961,23 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>32.7</v>
+        <v>29.2</v>
       </c>
       <c r="E69" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -2998,23 +2998,23 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>33.9</v>
+        <v>30.8</v>
       </c>
       <c r="E70" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>7.9</v>
+        <v>7.1</v>
       </c>
       <c r="H70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3035,23 +3035,23 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>32</v>
+        <v>27.9</v>
       </c>
       <c r="E71" t="n">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>4.4</v>
+        <v>1.5</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3072,23 +3072,23 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>31.5</v>
+        <v>28.6</v>
       </c>
       <c r="E72" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3109,23 +3109,23 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>32.8</v>
+        <v>28.2</v>
       </c>
       <c r="E73" t="n">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="F73" t="n">
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>4.9</v>
+        <v>2.5</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3146,23 +3146,23 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>34.9</v>
+        <v>31.2</v>
       </c>
       <c r="E74" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F74" t="n">
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3183,23 +3183,23 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>31</v>
+        <v>26.5</v>
       </c>
       <c r="E75" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>6.3</v>
+        <v>4.8</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3220,23 +3220,23 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>32.2</v>
+        <v>28.8</v>
       </c>
       <c r="E76" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>4.4</v>
+        <v>1.8</v>
       </c>
       <c r="H76" t="n">
         <v>0</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3257,23 +3257,23 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>33.8</v>
+        <v>30.1</v>
       </c>
       <c r="E77" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>4.1</v>
+        <v>5.7</v>
       </c>
       <c r="H77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3294,23 +3294,23 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>32.9</v>
+        <v>29</v>
       </c>
       <c r="E78" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="F78" t="n">
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>2.1</v>
+        <v>1.1</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>32.8</v>
+        <v>29.1</v>
       </c>
       <c r="E79" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>5.5</v>
+        <v>2.3</v>
       </c>
       <c r="H79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3368,23 +3368,23 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>31.3</v>
+        <v>27.6</v>
       </c>
       <c r="E80" t="n">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="F80" t="n">
         <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="H80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3405,23 +3405,23 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>33.1</v>
+        <v>29.2</v>
       </c>
       <c r="E81" t="n">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>4.6</v>
+        <v>3.8</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3442,23 +3442,23 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>31.4</v>
+        <v>27.3</v>
       </c>
       <c r="E82" t="n">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>6.6</v>
+        <v>4.4</v>
       </c>
       <c r="H82" t="n">
         <v>0</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3479,23 +3479,23 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>32.2</v>
+        <v>27.9</v>
       </c>
       <c r="E83" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="H83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3516,23 +3516,23 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>31.8</v>
+        <v>28.7</v>
       </c>
       <c r="E84" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>5.6</v>
+        <v>3.6</v>
       </c>
       <c r="H84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3553,23 +3553,23 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>32.3</v>
+        <v>28.3</v>
       </c>
       <c r="E85" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>9</v>
+        <v>3.8</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3590,23 +3590,23 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E86" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>5.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3627,23 +3627,23 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>31.9</v>
+        <v>27.9</v>
       </c>
       <c r="E87" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>8.699999999999999</v>
+        <v>5.4</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3664,23 +3664,23 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>31.5</v>
+        <v>28.4</v>
       </c>
       <c r="E88" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>5.5</v>
+        <v>3.2</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3701,23 +3701,23 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>31.1</v>
+        <v>28</v>
       </c>
       <c r="E89" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>6.5</v>
+        <v>0.7</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3738,23 +3738,23 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>32.4</v>
+        <v>28.6</v>
       </c>
       <c r="E90" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>4.9</v>
+        <v>3.4</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3775,23 +3775,23 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>32</v>
+        <v>28.4</v>
       </c>
       <c r="E91" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>3.4</v>
+        <v>1.9</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3812,23 +3812,23 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>31</v>
+        <v>26.9</v>
       </c>
       <c r="E92" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="F92" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>7.3</v>
+        <v>6</v>
       </c>
       <c r="H92" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3849,23 +3849,23 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>32.4</v>
+        <v>27.7</v>
       </c>
       <c r="E93" t="n">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="F93" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>6.7</v>
+        <v>4.6</v>
       </c>
       <c r="H93" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3886,23 +3886,23 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>31.1</v>
+        <v>27.2</v>
       </c>
       <c r="E94" t="n">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="F94" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>4.9</v>
+        <v>3.3</v>
       </c>
       <c r="H94" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3923,23 +3923,23 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>33.8</v>
+        <v>30.2</v>
       </c>
       <c r="E95" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
       <c r="H95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3960,23 +3960,23 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>30.8</v>
+        <v>26.8</v>
       </c>
       <c r="E96" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="F96" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>8.800000000000001</v>
+        <v>4.8</v>
       </c>
       <c r="H96" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -3997,23 +3997,23 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>33.5</v>
+        <v>29.8</v>
       </c>
       <c r="E97" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
       </c>
       <c r="G97" t="n">
-        <v>7.4</v>
+        <v>3.9</v>
       </c>
       <c r="H97" t="n">
         <v>0</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -4034,23 +4034,23 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>32.8</v>
+        <v>29.1</v>
       </c>
       <c r="E98" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
       </c>
       <c r="G98" t="n">
-        <v>4</v>
+        <v>4.4</v>
       </c>
       <c r="H98" t="n">
         <v>0</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-16T14:15</t>
+          <t>2026-09-16T19:15</t>
         </is>
       </c>
     </row>
@@ -4071,23 +4071,1244 @@
         </is>
       </c>
       <c r="D99" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="E99" t="n">
+        <v>72</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H99" t="n">
+        <v>1</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-09-16T19:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E100" t="n">
+        <v>63</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E101" t="n">
+        <v>63</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" t="n">
+        <v>6</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>32</v>
+      </c>
+      <c r="E102" t="n">
+        <v>57</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G102" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H102" t="n">
+        <v>51</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>40</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G103" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H103" t="n">
+        <v>51</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>31</v>
+      </c>
+      <c r="E104" t="n">
+        <v>63</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E105" t="n">
+        <v>64</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H105" t="n">
+        <v>1</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E106" t="n">
+        <v>60</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="E107" t="n">
+        <v>47</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E108" t="n">
+        <v>62</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
+        <v>5</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E109" t="n">
+        <v>61</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E110" t="n">
+        <v>58</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="E111" t="n">
+        <v>60</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H111" t="n">
+        <v>1</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="E112" t="n">
+        <v>62</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E113" t="n">
+        <v>60</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>9</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
         <v>32.3</v>
       </c>
-      <c r="E99" t="n">
+      <c r="E114" t="n">
+        <v>62</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H114" t="n">
+        <v>1</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E115" t="n">
+        <v>63</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="E116" t="n">
+        <v>48</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H116" t="n">
+        <v>1</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E117" t="n">
+        <v>64</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E118" t="n">
+        <v>55</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G118" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H118" t="n">
+        <v>51</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="E119" t="n">
+        <v>44</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H119" t="n">
+        <v>1</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E120" t="n">
+        <v>56</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E121" t="n">
+        <v>62</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="n">
+        <v>7</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E122" t="n">
+        <v>61</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E123" t="n">
+        <v>63</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E124" t="n">
+        <v>58</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="E125" t="n">
+        <v>53</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E126" t="n">
         <v>50</v>
       </c>
-      <c r="F99" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="H99" t="n">
-        <v>0</v>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>2026-09-16T14:15</t>
+      <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="E127" t="n">
+        <v>60</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H127" t="n">
+        <v>1</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="E128" t="n">
+        <v>52</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E129" t="n">
+        <v>59</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G129" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H129" t="n">
+        <v>51</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="E130" t="n">
+        <v>50</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H130" t="n">
+        <v>1</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="E131" t="n">
+        <v>55</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E132" t="n">
+        <v>57</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:15</t>
         </is>
       </c>
     </row>
@@ -4102,7 +5323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4304,29 +5525,29 @@
         <v>33</v>
       </c>
       <c r="D4" t="n">
-        <v>32.4</v>
+        <v>28.6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Nalgonda</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>35</v>
+        <v>31.2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Vikarabad</t>
+          <t>Kamareddy</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>30.8</v>
+        <v>26.5</v>
       </c>
       <c r="I4" t="n">
-        <v>52.7</v>
+        <v>71.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -4334,15 +5555,71 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Nagarkurnool</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="N4" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I5" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10.1</v>
       </c>
     </row>
   </sheetData>
@@ -4408,19 +5685,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>29.7</v>
+        <v>29.2</v>
       </c>
       <c r="D2" t="n">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="E2" t="n">
         <v>25.1</v>
       </c>
       <c r="F2" t="n">
-        <v>67.3</v>
+        <v>72</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -4438,13 +5715,13 @@
         <v>29.7</v>
       </c>
       <c r="D3" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="E3" t="n">
         <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>76</v>
+        <v>75.2</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -4462,19 +5739,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29.7</v>
+        <v>29.4</v>
       </c>
       <c r="D4" t="n">
-        <v>32.7</v>
+        <v>32</v>
       </c>
       <c r="E4" t="n">
         <v>24.9</v>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
+        <v>71.8</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -4489,19 +5766,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30.3</v>
+        <v>30.2</v>
       </c>
       <c r="D5" t="n">
-        <v>33.9</v>
+        <v>33.1</v>
       </c>
       <c r="E5" t="n">
         <v>24.8</v>
       </c>
       <c r="F5" t="n">
-        <v>54.7</v>
+        <v>53.2</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
@@ -4516,16 +5793,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>29.6</v>
+        <v>28.9</v>
       </c>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E6" t="n">
         <v>25.7</v>
       </c>
       <c r="F6" t="n">
-        <v>67.3</v>
+        <v>72.8</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -4543,16 +5820,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>28.7</v>
       </c>
       <c r="D7" t="n">
-        <v>31.5</v>
+        <v>31</v>
       </c>
       <c r="E7" t="n">
         <v>24.4</v>
       </c>
       <c r="F7" t="n">
-        <v>68.7</v>
+        <v>71.8</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -4570,16 +5847,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.7</v>
+        <v>29.2</v>
       </c>
       <c r="D8" t="n">
-        <v>32.8</v>
+        <v>32.5</v>
       </c>
       <c r="E8" t="n">
         <v>24.6</v>
       </c>
       <c r="F8" t="n">
-        <v>72</v>
+        <v>76.2</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -4597,16 +5874,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>32</v>
+        <v>31.5</v>
       </c>
       <c r="D9" t="n">
-        <v>34.9</v>
+        <v>33.8</v>
       </c>
       <c r="E9" t="n">
         <v>27.4</v>
       </c>
       <c r="F9" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -4624,16 +5901,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>27.4</v>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>30.2</v>
       </c>
       <c r="E10" t="n">
         <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>66.7</v>
+        <v>72.5</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -4651,16 +5928,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29.9</v>
+        <v>29.5</v>
       </c>
       <c r="D11" t="n">
-        <v>32.2</v>
+        <v>31.8</v>
       </c>
       <c r="E11" t="n">
         <v>26</v>
       </c>
       <c r="F11" t="n">
-        <v>68.3</v>
+        <v>71.5</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -4678,16 +5955,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30.6</v>
+        <v>30.4</v>
       </c>
       <c r="D12" t="n">
-        <v>33.8</v>
+        <v>33.3</v>
       </c>
       <c r="E12" t="n">
         <v>25.5</v>
       </c>
       <c r="F12" t="n">
-        <v>69.3</v>
+        <v>70.8</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -4705,16 +5982,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>29.9</v>
+        <v>29.5</v>
       </c>
       <c r="D13" t="n">
-        <v>32.9</v>
+        <v>32.1</v>
       </c>
       <c r="E13" t="n">
         <v>25.3</v>
       </c>
       <c r="F13" t="n">
-        <v>69.7</v>
+        <v>73</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -4732,16 +6009,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29.8</v>
+        <v>29.5</v>
       </c>
       <c r="D14" t="n">
-        <v>32.8</v>
+        <v>32.2</v>
       </c>
       <c r="E14" t="n">
         <v>24.9</v>
       </c>
       <c r="F14" t="n">
-        <v>72.7</v>
+        <v>75</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -4759,16 +6036,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.7</v>
+        <v>28.2</v>
       </c>
       <c r="D15" t="n">
-        <v>31.3</v>
+        <v>30.6</v>
       </c>
       <c r="E15" t="n">
         <v>24.3</v>
       </c>
       <c r="F15" t="n">
-        <v>60.3</v>
+        <v>65.8</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -4786,16 +6063,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.6</v>
+        <v>30.1</v>
       </c>
       <c r="D16" t="n">
-        <v>33.1</v>
+        <v>32.3</v>
       </c>
       <c r="E16" t="n">
         <v>26.8</v>
       </c>
       <c r="F16" t="n">
-        <v>70.7</v>
+        <v>74</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -4813,16 +6090,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>28.6</v>
+        <v>28</v>
       </c>
       <c r="D17" t="n">
-        <v>31.4</v>
+        <v>30.5</v>
       </c>
       <c r="E17" t="n">
         <v>24.3</v>
       </c>
       <c r="F17" t="n">
-        <v>66.7</v>
+        <v>71</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -4840,16 +6117,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>27.9</v>
       </c>
       <c r="D18" t="n">
-        <v>32.2</v>
+        <v>31.9</v>
       </c>
       <c r="E18" t="n">
         <v>23.9</v>
       </c>
       <c r="F18" t="n">
-        <v>64.5</v>
+        <v>64.7</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -4867,16 +6144,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28.9</v>
+        <v>28.8</v>
       </c>
       <c r="D19" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="E19" t="n">
         <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>75.7</v>
+        <v>76</v>
       </c>
       <c r="G19" t="n">
         <v>0.1</v>
@@ -4894,19 +6171,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.4</v>
+        <v>28.8</v>
       </c>
       <c r="D20" t="n">
-        <v>32.3</v>
+        <v>31.2</v>
       </c>
       <c r="E20" t="n">
         <v>24.7</v>
       </c>
       <c r="F20" t="n">
-        <v>62.7</v>
+        <v>65</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="21">
@@ -4921,16 +6198,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="D21" t="n">
-        <v>35</v>
+        <v>34.6</v>
       </c>
       <c r="E21" t="n">
         <v>25.7</v>
       </c>
       <c r="F21" t="n">
-        <v>59.3</v>
+        <v>59.8</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -4948,16 +6225,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>29.4</v>
+        <v>28.8</v>
       </c>
       <c r="D22" t="n">
-        <v>31.9</v>
+        <v>31.3</v>
       </c>
       <c r="E22" t="n">
         <v>25</v>
       </c>
       <c r="F22" t="n">
-        <v>57.7</v>
+        <v>61</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -4975,16 +6252,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.8</v>
+        <v>28.5</v>
       </c>
       <c r="D23" t="n">
-        <v>31.5</v>
+        <v>30.6</v>
       </c>
       <c r="E23" t="n">
         <v>24.4</v>
       </c>
       <c r="F23" t="n">
-        <v>69.3</v>
+        <v>71.8</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -5002,7 +6279,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.7</v>
+        <v>28.5</v>
       </c>
       <c r="D24" t="n">
         <v>31.1</v>
@@ -5011,7 +6288,7 @@
         <v>24.7</v>
       </c>
       <c r="F24" t="n">
-        <v>66</v>
+        <v>69.8</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -5029,16 +6306,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.9</v>
+        <v>29.4</v>
       </c>
       <c r="D25" t="n">
-        <v>32.4</v>
+        <v>31.8</v>
       </c>
       <c r="E25" t="n">
         <v>25.9</v>
       </c>
       <c r="F25" t="n">
-        <v>71.7</v>
+        <v>74.8</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -5056,16 +6333,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>29.4</v>
+        <v>29.1</v>
       </c>
       <c r="D26" t="n">
-        <v>32</v>
+        <v>31.7</v>
       </c>
       <c r="E26" t="n">
         <v>25.2</v>
       </c>
       <c r="F26" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -5083,19 +6360,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.6</v>
+        <v>28.1</v>
       </c>
       <c r="D27" t="n">
-        <v>31</v>
+        <v>30.7</v>
       </c>
       <c r="E27" t="n">
         <v>24.2</v>
       </c>
       <c r="F27" t="n">
-        <v>61.7</v>
+        <v>64</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28">
@@ -5110,19 +6387,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29.3</v>
+        <v>28.8</v>
       </c>
       <c r="D28" t="n">
-        <v>32.4</v>
+        <v>31.8</v>
       </c>
       <c r="E28" t="n">
         <v>24.5</v>
       </c>
       <c r="F28" t="n">
-        <v>58.3</v>
+        <v>62</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29">
@@ -5137,19 +6414,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28.4</v>
+        <v>28</v>
       </c>
       <c r="D29" t="n">
-        <v>31.1</v>
+        <v>30.7</v>
       </c>
       <c r="E29" t="n">
         <v>24.4</v>
       </c>
       <c r="F29" t="n">
-        <v>66.7</v>
+        <v>71.2</v>
       </c>
       <c r="G29" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="30">
@@ -5164,16 +6441,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30.7</v>
+        <v>30.5</v>
       </c>
       <c r="D30" t="n">
-        <v>33.8</v>
+        <v>33.7</v>
       </c>
       <c r="E30" t="n">
         <v>25.4</v>
       </c>
       <c r="F30" t="n">
-        <v>66.7</v>
+        <v>67</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -5191,16 +6468,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>28.2</v>
+        <v>27.6</v>
       </c>
       <c r="D31" t="n">
-        <v>30.8</v>
+        <v>29.9</v>
       </c>
       <c r="E31" t="n">
         <v>23.9</v>
       </c>
       <c r="F31" t="n">
-        <v>62</v>
+        <v>65.8</v>
       </c>
       <c r="G31" t="n">
         <v>0.1</v>
@@ -5218,16 +6495,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30.6</v>
+        <v>30.1</v>
       </c>
       <c r="D32" t="n">
-        <v>33.5</v>
+        <v>32.4</v>
       </c>
       <c r="E32" t="n">
         <v>26.4</v>
       </c>
       <c r="F32" t="n">
-        <v>54.3</v>
+        <v>55.8</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -5245,16 +6522,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>29.7</v>
+        <v>29.4</v>
       </c>
       <c r="D33" t="n">
-        <v>32.8</v>
+        <v>32.3</v>
       </c>
       <c r="E33" t="n">
         <v>24.7</v>
       </c>
       <c r="F33" t="n">
-        <v>70.3</v>
+        <v>70.8</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -5272,16 +6549,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>29.5</v>
+        <v>29</v>
       </c>
       <c r="D34" t="n">
-        <v>32.3</v>
+        <v>31.6</v>
       </c>
       <c r="E34" t="n">
         <v>24.5</v>
       </c>
       <c r="F34" t="n">
-        <v>62.7</v>
+        <v>66.8</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update weather analytics project
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I132"/>
+  <dimension ref="A1:I165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4108,23 +4108,23 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>30.5</v>
+        <v>25.3</v>
       </c>
       <c r="E100" t="n">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G100" t="n">
-        <v>3.4</v>
+        <v>7.3</v>
       </c>
       <c r="H100" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4145,23 +4145,23 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>31.8</v>
+        <v>28.5</v>
       </c>
       <c r="E101" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="F101" t="n">
         <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>5.9</v>
+        <v>2.1</v>
       </c>
       <c r="H101" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4182,23 +4182,23 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>33.2</v>
+        <v>28.7</v>
       </c>
       <c r="E102" t="n">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="H102" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4219,23 +4219,23 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>33.7</v>
+        <v>29.7</v>
       </c>
       <c r="E103" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="F103" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G103" t="n">
-        <v>8.5</v>
+        <v>1.8</v>
       </c>
       <c r="H103" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4256,23 +4256,23 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>32.1</v>
+        <v>26.7</v>
       </c>
       <c r="E104" t="n">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
       <c r="H104" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4293,23 +4293,23 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>31.9</v>
+        <v>26.6</v>
       </c>
       <c r="E105" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
       </c>
       <c r="G105" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="H105" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4330,23 +4330,23 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>31.2</v>
+        <v>27.7</v>
       </c>
       <c r="E106" t="n">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="F106" t="n">
         <v>0</v>
       </c>
       <c r="G106" t="n">
-        <v>5.2</v>
+        <v>1.5</v>
       </c>
       <c r="H106" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4367,23 +4367,23 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>35.6</v>
+        <v>25.8</v>
       </c>
       <c r="E107" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="F107" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="G107" t="n">
-        <v>10.6</v>
+        <v>19.8</v>
       </c>
       <c r="H107" t="n">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4404,23 +4404,23 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>30.8</v>
+        <v>25.5</v>
       </c>
       <c r="E108" t="n">
-        <v>57</v>
+        <v>87</v>
       </c>
       <c r="F108" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="G108" t="n">
-        <v>7.3</v>
+        <v>2.9</v>
       </c>
       <c r="H108" t="n">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>32.3</v>
+        <v>27.2</v>
       </c>
       <c r="E109" t="n">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="H109" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4478,23 +4478,23 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>34</v>
+        <v>29.4</v>
       </c>
       <c r="E110" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="F110" t="n">
         <v>0</v>
       </c>
       <c r="G110" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4515,23 +4515,23 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>33.4</v>
+        <v>26.7</v>
       </c>
       <c r="E111" t="n">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="F111" t="n">
         <v>0</v>
       </c>
       <c r="G111" t="n">
-        <v>1.9</v>
+        <v>3.3</v>
       </c>
       <c r="H111" t="n">
         <v>1</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4552,23 +4552,23 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>32.7</v>
+        <v>28.5</v>
       </c>
       <c r="E112" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="F112" t="n">
         <v>0</v>
       </c>
       <c r="G112" t="n">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="H112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4589,23 +4589,23 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>31.8</v>
+        <v>26.6</v>
       </c>
       <c r="E113" t="n">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="F113" t="n">
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>9.5</v>
+        <v>4.2</v>
       </c>
       <c r="H113" t="n">
         <v>1</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4626,23 +4626,23 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>31.8</v>
+        <v>28.2</v>
       </c>
       <c r="E114" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="F114" t="n">
         <v>0</v>
       </c>
       <c r="G114" t="n">
-        <v>5.3</v>
+        <v>2.4</v>
       </c>
       <c r="H114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4663,23 +4663,23 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>31.4</v>
+        <v>25.4</v>
       </c>
       <c r="E115" t="n">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="F115" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G115" t="n">
-        <v>7.8</v>
+        <v>3.8</v>
       </c>
       <c r="H115" t="n">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4700,23 +4700,23 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>32.2</v>
+        <v>26.6</v>
       </c>
       <c r="E116" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="F116" t="n">
         <v>0</v>
       </c>
       <c r="G116" t="n">
-        <v>8.6</v>
+        <v>3.9</v>
       </c>
       <c r="H116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4737,23 +4737,23 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31.3</v>
+        <v>27.9</v>
       </c>
       <c r="E117" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="F117" t="n">
         <v>0</v>
       </c>
       <c r="G117" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="H117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4774,23 +4774,23 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>32.8</v>
+        <v>28</v>
       </c>
       <c r="E118" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="F118" t="n">
         <v>0</v>
       </c>
       <c r="G118" t="n">
-        <v>10.9</v>
+        <v>4.4</v>
       </c>
       <c r="H118" t="n">
         <v>0</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4811,23 +4811,23 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>36.2</v>
+        <v>30.4</v>
       </c>
       <c r="E119" t="n">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
       </c>
       <c r="G119" t="n">
-        <v>5.2</v>
+        <v>3.5</v>
       </c>
       <c r="H119" t="n">
         <v>1</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4848,23 +4848,23 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>32.6</v>
+        <v>27.2</v>
       </c>
       <c r="E120" t="n">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="F120" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G120" t="n">
-        <v>10.1</v>
+        <v>4.3</v>
       </c>
       <c r="H120" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4885,23 +4885,23 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>30.7</v>
+        <v>26.4</v>
       </c>
       <c r="E121" t="n">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="F121" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G121" t="n">
-        <v>10.2</v>
+        <v>9.9</v>
       </c>
       <c r="H121" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4922,23 +4922,23 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>31.8</v>
+        <v>24.2</v>
       </c>
       <c r="E122" t="n">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="F122" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G122" t="n">
-        <v>4.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H122" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4959,23 +4959,23 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>31.8</v>
+        <v>27.2</v>
       </c>
       <c r="E123" t="n">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -4996,23 +4996,23 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>32.3</v>
+        <v>26.3</v>
       </c>
       <c r="E124" t="n">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H124" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5033,23 +5033,23 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>31.2</v>
+        <v>26.3</v>
       </c>
       <c r="E125" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="F125" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G125" t="n">
-        <v>10.3</v>
+        <v>0.7</v>
       </c>
       <c r="H125" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5070,23 +5070,23 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32.2</v>
+        <v>26</v>
       </c>
       <c r="E126" t="n">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="F126" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>9.199999999999999</v>
+        <v>5.6</v>
       </c>
       <c r="H126" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5107,23 +5107,23 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E127" t="n">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F127" t="n">
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>6.1</v>
+        <v>3.2</v>
       </c>
       <c r="H127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5144,23 +5144,23 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>34.6</v>
+        <v>29.7</v>
       </c>
       <c r="E128" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="H128" t="n">
         <v>1</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5181,23 +5181,23 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>30.8</v>
+        <v>26.2</v>
       </c>
       <c r="E129" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="F129" t="n">
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>10.7</v>
+        <v>3.6</v>
       </c>
       <c r="H129" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5218,23 +5218,23 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>34.1</v>
+        <v>28.1</v>
       </c>
       <c r="E130" t="n">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="F130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G130" t="n">
-        <v>9.4</v>
+        <v>1.1</v>
       </c>
       <c r="H130" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5255,23 +5255,23 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>33.6</v>
+        <v>29</v>
       </c>
       <c r="E131" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="F131" t="n">
         <v>0</v>
       </c>
       <c r="G131" t="n">
-        <v>1.7</v>
+        <v>2.7</v>
       </c>
       <c r="H131" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-09-17T14:15</t>
+          <t>2026-09-17T21:45</t>
         </is>
       </c>
     </row>
@@ -5292,23 +5292,1244 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>32.6</v>
+        <v>27.1</v>
       </c>
       <c r="E132" t="n">
+        <v>76</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H132" t="n">
+        <v>3</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-09-17T21:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="E133" t="n">
+        <v>66</v>
+      </c>
+      <c r="F133" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G133" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H133" t="n">
+        <v>1</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E134" t="n">
+        <v>60</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G134" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H134" t="n">
+        <v>1</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E135" t="n">
+        <v>63</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G135" t="n">
+        <v>12</v>
+      </c>
+      <c r="H135" t="n">
+        <v>1</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E136" t="n">
+        <v>59</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G136" t="n">
+        <v>12</v>
+      </c>
+      <c r="H136" t="n">
+        <v>1</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>30</v>
+      </c>
+      <c r="E137" t="n">
+        <v>65</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G137" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H137" t="n">
+        <v>1</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="E138" t="n">
+        <v>58</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G138" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="H138" t="n">
+        <v>1</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>31</v>
+      </c>
+      <c r="E139" t="n">
+        <v>61</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G139" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="H139" t="n">
+        <v>1</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="E140" t="n">
+        <v>54</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G140" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H140" t="n">
+        <v>1</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E141" t="n">
+        <v>65</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G141" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H141" t="n">
+        <v>1</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E142" t="n">
+        <v>64</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G142" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H142" t="n">
+        <v>1</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="E143" t="n">
+        <v>58</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G143" t="n">
+        <v>15</v>
+      </c>
+      <c r="H143" t="n">
+        <v>1</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="E144" t="n">
+        <v>68</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G144" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H144" t="n">
+        <v>1</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E145" t="n">
+        <v>60</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G145" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H145" t="n">
+        <v>1</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E146" t="n">
+        <v>56</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G146" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H146" t="n">
+        <v>1</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="E147" t="n">
+        <v>66</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1</v>
+      </c>
+      <c r="G147" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H147" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="E148" t="n">
+        <v>62</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G148" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H148" t="n">
+        <v>1</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="E149" t="n">
+        <v>61</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G149" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H149" t="n">
+        <v>1</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E150" t="n">
+        <v>66</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G150" t="n">
+        <v>11</v>
+      </c>
+      <c r="H150" t="n">
+        <v>1</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E151" t="n">
+        <v>57</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G151" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H151" t="n">
+        <v>1</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E152" t="n">
+        <v>57</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G152" t="n">
+        <v>14</v>
+      </c>
+      <c r="H152" t="n">
+        <v>1</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-09-18T12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E153" t="n">
+        <v>59</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H153" t="n">
+        <v>1</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E154" t="n">
+        <v>70</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="E155" t="n">
+        <v>76</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H155" t="n">
+        <v>2</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E156" t="n">
+        <v>70</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G156" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H156" t="n">
         <v>51</v>
       </c>
-      <c r="F132" t="n">
-        <v>0</v>
-      </c>
-      <c r="G132" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="H132" t="n">
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E157" t="n">
+        <v>67</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H157" t="n">
+        <v>2</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="E158" t="n">
+        <v>64</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H158" t="n">
         <v>1</v>
       </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>2026-09-17T14:15</t>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="E159" t="n">
+        <v>65</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H159" t="n">
+        <v>3</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="E160" t="n">
+        <v>70</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
+        <v>11</v>
+      </c>
+      <c r="H160" t="n">
+        <v>2</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="E161" t="n">
+        <v>55</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="E162" t="n">
+        <v>66</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G162" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H162" t="n">
+        <v>51</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E163" t="n">
+        <v>54</v>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="H163" t="n">
+        <v>2</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E164" t="n">
+        <v>63</v>
+      </c>
+      <c r="F164" t="n">
+        <v>0</v>
+      </c>
+      <c r="G164" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H164" t="n">
+        <v>1</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E165" t="n">
+        <v>62</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H165" t="n">
+        <v>2</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>2026-09-18T11:15</t>
         </is>
       </c>
     </row>
@@ -5323,7 +6544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5581,7 +6802,7 @@
         <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>32.4</v>
+        <v>27.2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -5589,37 +6810,93 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>36.2</v>
+        <v>30.4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Adilabad</t>
+          <t>Nizamabad</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>30.5</v>
+        <v>24.2</v>
       </c>
       <c r="I5" t="n">
-        <v>56.2</v>
+        <v>80.8</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7</v>
+        <v>4.6</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Nirmal</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Nagarkurnool</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>10.9</v>
+        <v>19.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -5685,7 +6962,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28.9</v>
+        <v>28</v>
       </c>
       <c r="D2" t="n">
         <v>31.4</v>
@@ -5694,10 +6971,10 @@
         <v>25.1</v>
       </c>
       <c r="F2" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3">
@@ -5712,19 +6989,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>29.5</v>
+        <v>29.3</v>
       </c>
       <c r="D3" t="n">
-        <v>31.8</v>
+        <v>31.6</v>
       </c>
       <c r="E3" t="n">
         <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>76.5</v>
+        <v>76.2</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -5739,19 +7016,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29.7</v>
+        <v>29</v>
       </c>
       <c r="D4" t="n">
-        <v>33.2</v>
+        <v>31.5</v>
       </c>
       <c r="E4" t="n">
         <v>24.9</v>
       </c>
       <c r="F4" t="n">
-        <v>71.5</v>
+        <v>75.2</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
@@ -5766,19 +7043,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30.4</v>
+        <v>29.7</v>
       </c>
       <c r="D5" t="n">
-        <v>33.7</v>
+        <v>32.1</v>
       </c>
       <c r="E5" t="n">
         <v>24.8</v>
       </c>
       <c r="F5" t="n">
-        <v>53.5</v>
+        <v>58.2</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
@@ -5793,19 +7070,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>29.2</v>
+        <v>28.3</v>
       </c>
       <c r="D6" t="n">
-        <v>32.1</v>
+        <v>31</v>
       </c>
       <c r="E6" t="n">
         <v>25.7</v>
       </c>
       <c r="F6" t="n">
-        <v>72.5</v>
+        <v>77.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
@@ -5820,19 +7097,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>28.4</v>
       </c>
       <c r="D7" t="n">
-        <v>31.9</v>
+        <v>31.3</v>
       </c>
       <c r="E7" t="n">
         <v>24.4</v>
       </c>
       <c r="F7" t="n">
-        <v>70.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
@@ -5847,7 +7124,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.9</v>
+        <v>28.6</v>
       </c>
       <c r="D8" t="n">
         <v>31.6</v>
@@ -5856,10 +7133,10 @@
         <v>24.6</v>
       </c>
       <c r="F8" t="n">
-        <v>77.5</v>
+        <v>77.8</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9">
@@ -5874,19 +7151,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>32</v>
+        <v>29.8</v>
       </c>
       <c r="D9" t="n">
-        <v>35.6</v>
+        <v>33.8</v>
       </c>
       <c r="E9" t="n">
-        <v>27.4</v>
+        <v>25.8</v>
       </c>
       <c r="F9" t="n">
-        <v>49</v>
+        <v>58.2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
@@ -5901,19 +7178,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.6</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>30.8</v>
+        <v>29.9</v>
       </c>
       <c r="E10" t="n">
         <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>71.2</v>
+        <v>76</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="11">
@@ -5928,19 +7205,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29.6</v>
+        <v>28.7</v>
       </c>
       <c r="D11" t="n">
-        <v>32.3</v>
+        <v>31.5</v>
       </c>
       <c r="E11" t="n">
         <v>26</v>
       </c>
       <c r="F11" t="n">
-        <v>71.8</v>
+        <v>76</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12">
@@ -5955,19 +7232,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30.5</v>
+        <v>29.9</v>
       </c>
       <c r="D12" t="n">
-        <v>34</v>
+        <v>32.5</v>
       </c>
       <c r="E12" t="n">
         <v>25.5</v>
       </c>
       <c r="F12" t="n">
-        <v>69.5</v>
+        <v>71.8</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13">
@@ -5982,19 +7259,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>29.8</v>
+        <v>28.3</v>
       </c>
       <c r="D13" t="n">
-        <v>33.4</v>
+        <v>31.6</v>
       </c>
       <c r="E13" t="n">
         <v>25.3</v>
       </c>
       <c r="F13" t="n">
-        <v>72</v>
+        <v>79.2</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="14">
@@ -6009,19 +7286,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29.6</v>
+        <v>29.1</v>
       </c>
       <c r="D14" t="n">
-        <v>32.7</v>
+        <v>31.7</v>
       </c>
       <c r="E14" t="n">
         <v>24.9</v>
       </c>
       <c r="F14" t="n">
-        <v>75</v>
+        <v>76.2</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="15">
@@ -6036,19 +7313,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.6</v>
+        <v>28</v>
       </c>
       <c r="D15" t="n">
-        <v>31.8</v>
+        <v>30.9</v>
       </c>
       <c r="E15" t="n">
         <v>24.3</v>
       </c>
       <c r="F15" t="n">
-        <v>63.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="16">
@@ -6063,7 +7340,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30</v>
+        <v>29.2</v>
       </c>
       <c r="D16" t="n">
         <v>32</v>
@@ -6072,10 +7349,10 @@
         <v>26.8</v>
       </c>
       <c r="F16" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -6090,19 +7367,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="D17" t="n">
-        <v>31.4</v>
+        <v>30.7</v>
       </c>
       <c r="E17" t="n">
         <v>24.3</v>
       </c>
       <c r="F17" t="n">
-        <v>69.5</v>
+        <v>73.8</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="18">
@@ -6117,19 +7394,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>27.2</v>
       </c>
       <c r="D18" t="n">
-        <v>32.2</v>
+        <v>30.6</v>
       </c>
       <c r="E18" t="n">
         <v>23.9</v>
       </c>
       <c r="F18" t="n">
-        <v>64.3</v>
+        <v>70</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19">
@@ -6144,19 +7421,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28.7</v>
+        <v>28.4</v>
       </c>
       <c r="D19" t="n">
-        <v>31.3</v>
+        <v>30.9</v>
       </c>
       <c r="E19" t="n">
         <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>76.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -6171,19 +7448,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="D20" t="n">
-        <v>32.8</v>
+        <v>31.2</v>
       </c>
       <c r="E20" t="n">
         <v>24.7</v>
       </c>
       <c r="F20" t="n">
-        <v>63.5</v>
+        <v>65.2</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="21">
@@ -6198,19 +7475,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.6</v>
+        <v>30.4</v>
       </c>
       <c r="D21" t="n">
-        <v>36.2</v>
+        <v>33.6</v>
       </c>
       <c r="E21" t="n">
         <v>25.7</v>
       </c>
       <c r="F21" t="n">
-        <v>59.5</v>
+        <v>63</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="22">
@@ -6225,19 +7502,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>29.2</v>
+        <v>28.4</v>
       </c>
       <c r="D22" t="n">
-        <v>32.6</v>
+        <v>31.3</v>
       </c>
       <c r="E22" t="n">
         <v>25</v>
       </c>
       <c r="F22" t="n">
-        <v>59.2</v>
+        <v>64</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="23">
@@ -6252,19 +7529,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.5</v>
+        <v>27.9</v>
       </c>
       <c r="D23" t="n">
-        <v>30.7</v>
+        <v>30.6</v>
       </c>
       <c r="E23" t="n">
         <v>24.4</v>
       </c>
       <c r="F23" t="n">
-        <v>72.8</v>
+        <v>76</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="24">
@@ -6279,19 +7556,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.7</v>
+        <v>27</v>
       </c>
       <c r="D24" t="n">
-        <v>31.8</v>
+        <v>30.2</v>
       </c>
       <c r="E24" t="n">
-        <v>24.7</v>
+        <v>24.2</v>
       </c>
       <c r="F24" t="n">
-        <v>69.5</v>
+        <v>78.2</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25">
@@ -6306,19 +7583,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.4</v>
+        <v>28.7</v>
       </c>
       <c r="D25" t="n">
-        <v>31.8</v>
+        <v>31.5</v>
       </c>
       <c r="E25" t="n">
         <v>25.9</v>
       </c>
       <c r="F25" t="n">
-        <v>75.5</v>
+        <v>79.8</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -6333,16 +7610,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>29.2</v>
+        <v>28.2</v>
       </c>
       <c r="D26" t="n">
-        <v>32.3</v>
+        <v>31.1</v>
       </c>
       <c r="E26" t="n">
         <v>25.2</v>
       </c>
       <c r="F26" t="n">
-        <v>72.5</v>
+        <v>76.2</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -6360,19 +7637,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="D27" t="n">
-        <v>31.2</v>
+        <v>30.5</v>
       </c>
       <c r="E27" t="n">
         <v>24.2</v>
       </c>
       <c r="F27" t="n">
-        <v>64</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28">
@@ -6387,19 +7664,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.9</v>
+        <v>27.7</v>
       </c>
       <c r="D28" t="n">
-        <v>32.2</v>
+        <v>31.1</v>
       </c>
       <c r="E28" t="n">
         <v>24.5</v>
       </c>
       <c r="F28" t="n">
-        <v>61.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29">
@@ -6414,16 +7691,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28.1</v>
+        <v>27.3</v>
       </c>
       <c r="D29" t="n">
-        <v>31</v>
+        <v>29.8</v>
       </c>
       <c r="E29" t="n">
         <v>24.4</v>
       </c>
       <c r="F29" t="n">
-        <v>72</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G29" t="n">
         <v>0.1</v>
@@ -6441,16 +7718,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30.8</v>
+        <v>30.2</v>
       </c>
       <c r="D30" t="n">
-        <v>34.6</v>
+        <v>33.1</v>
       </c>
       <c r="E30" t="n">
         <v>25.4</v>
       </c>
       <c r="F30" t="n">
-        <v>66.5</v>
+        <v>68.2</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -6468,19 +7745,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>27.8</v>
+        <v>27.1</v>
       </c>
       <c r="D31" t="n">
-        <v>30.8</v>
+        <v>29.8</v>
       </c>
       <c r="E31" t="n">
         <v>23.9</v>
       </c>
       <c r="F31" t="n">
-        <v>65.2</v>
+        <v>68.8</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="32">
@@ -6495,19 +7772,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30.6</v>
+        <v>29.6</v>
       </c>
       <c r="D32" t="n">
-        <v>34.1</v>
+        <v>31.9</v>
       </c>
       <c r="E32" t="n">
         <v>26.4</v>
       </c>
       <c r="F32" t="n">
-        <v>54</v>
+        <v>58.4</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -6522,16 +7799,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>29.8</v>
+        <v>29.2</v>
       </c>
       <c r="D33" t="n">
-        <v>33.6</v>
+        <v>31.7</v>
       </c>
       <c r="E33" t="n">
         <v>24.7</v>
       </c>
       <c r="F33" t="n">
-        <v>70.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -6549,16 +7826,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>29.3</v>
+        <v>28.5</v>
       </c>
       <c r="D34" t="n">
-        <v>32.6</v>
+        <v>31.6</v>
       </c>
       <c r="E34" t="n">
         <v>24.5</v>
       </c>
       <c r="F34" t="n">
-        <v>65.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix dashboard to show all districts
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I693"/>
+  <dimension ref="A1:I628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22409,12 +22409,12 @@
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Adilabad</t>
+          <t>Mahabubabad</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -22423,35 +22423,35 @@
         </is>
       </c>
       <c r="D595" t="n">
-        <v>24.3</v>
+        <v>31.2</v>
       </c>
       <c r="E595" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="F595" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="G595" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="H595" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="I595" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T12:00</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>Bhadradri Kothagudem</t>
+          <t>Adilabad</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -22460,35 +22460,35 @@
         </is>
       </c>
       <c r="D596" t="n">
-        <v>25.2</v>
+        <v>29.7</v>
       </c>
       <c r="E596" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="F596" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G596" t="n">
-        <v>18.6</v>
+        <v>20</v>
       </c>
       <c r="H596" t="n">
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="I596" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>Hanumakonda</t>
+          <t>Bhadradri Kothagudem</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -22497,35 +22497,35 @@
         </is>
       </c>
       <c r="D597" t="n">
-        <v>24.2</v>
+        <v>25.1</v>
       </c>
       <c r="E597" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F597" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="G597" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="H597" t="n">
         <v>80</v>
       </c>
       <c r="I597" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Hanumakonda</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -22534,35 +22534,35 @@
         </is>
       </c>
       <c r="D598" t="n">
-        <v>23.1</v>
+        <v>25.8</v>
       </c>
       <c r="E598" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F598" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G598" t="n">
-        <v>14.4</v>
+        <v>17.9</v>
       </c>
       <c r="H598" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I598" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>Jagtial</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -22571,35 +22571,35 @@
         </is>
       </c>
       <c r="D599" t="n">
-        <v>24.4</v>
+        <v>27.3</v>
       </c>
       <c r="E599" t="n">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="F599" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G599" t="n">
-        <v>16.4</v>
+        <v>17.4</v>
       </c>
       <c r="H599" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I599" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>Jangaon</t>
+          <t>Jagtial</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -22608,35 +22608,35 @@
         </is>
       </c>
       <c r="D600" t="n">
-        <v>24.2</v>
+        <v>28.1</v>
       </c>
       <c r="E600" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F600" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G600" t="n">
-        <v>22.4</v>
+        <v>18.6</v>
       </c>
       <c r="H600" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I600" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>Jayashankar Bhupalpally</t>
+          <t>Jangaon</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -22645,35 +22645,35 @@
         </is>
       </c>
       <c r="D601" t="n">
-        <v>24.1</v>
+        <v>26.7</v>
       </c>
       <c r="E601" t="n">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="F601" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G601" t="n">
-        <v>15.8</v>
+        <v>26.7</v>
       </c>
       <c r="H601" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I601" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Jogulamba Gadwal</t>
+          <t>Jayashankar Bhupalpally</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -22682,35 +22682,35 @@
         </is>
       </c>
       <c r="D602" t="n">
-        <v>24.7</v>
+        <v>26.3</v>
       </c>
       <c r="E602" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F602" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G602" t="n">
-        <v>20</v>
+        <v>15.3</v>
       </c>
       <c r="H602" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I602" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>Kamareddy</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
@@ -22719,35 +22719,35 @@
         </is>
       </c>
       <c r="D603" t="n">
-        <v>23</v>
+        <v>30.3</v>
       </c>
       <c r="E603" t="n">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="F603" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G603" t="n">
-        <v>19.2</v>
+        <v>26.6</v>
       </c>
       <c r="H603" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="I603" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>Karimnagar</t>
+          <t>Kamareddy</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
@@ -22756,35 +22756,35 @@
         </is>
       </c>
       <c r="D604" t="n">
-        <v>24.4</v>
+        <v>26.4</v>
       </c>
       <c r="E604" t="n">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="F604" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G604" t="n">
-        <v>14.9</v>
+        <v>22.3</v>
       </c>
       <c r="H604" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I604" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>Khammam</t>
+          <t>Karimnagar</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -22793,35 +22793,35 @@
         </is>
       </c>
       <c r="D605" t="n">
-        <v>25.7</v>
+        <v>27.3</v>
       </c>
       <c r="E605" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="F605" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="G605" t="n">
-        <v>18.6</v>
+        <v>19.7</v>
       </c>
       <c r="H605" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="I605" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>Kumuram Bheem Asifabad</t>
+          <t>Khammam</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -22830,35 +22830,35 @@
         </is>
       </c>
       <c r="D606" t="n">
-        <v>24.6</v>
+        <v>26.3</v>
       </c>
       <c r="E606" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F606" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G606" t="n">
-        <v>15.1</v>
+        <v>21.1</v>
       </c>
       <c r="H606" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I606" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>Mahabubabad</t>
+          <t>Kumuram Bheem Asifabad</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -22867,35 +22867,35 @@
         </is>
       </c>
       <c r="D607" t="n">
-        <v>25.2</v>
+        <v>28.9</v>
       </c>
       <c r="E607" t="n">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F607" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G607" t="n">
-        <v>20.8</v>
+        <v>19.6</v>
       </c>
       <c r="H607" t="n">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="I607" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>Mahbubnagar</t>
+          <t>Mahabubabad</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -22904,35 +22904,35 @@
         </is>
       </c>
       <c r="D608" t="n">
-        <v>22.4</v>
+        <v>25.4</v>
       </c>
       <c r="E608" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F608" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G608" t="n">
-        <v>15.3</v>
+        <v>23.4</v>
       </c>
       <c r="H608" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I608" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Mancherial</t>
+          <t>Mahbubnagar</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
@@ -22941,35 +22941,35 @@
         </is>
       </c>
       <c r="D609" t="n">
-        <v>25</v>
+        <v>28.2</v>
       </c>
       <c r="E609" t="n">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="F609" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G609" t="n">
-        <v>11.9</v>
+        <v>23.7</v>
       </c>
       <c r="H609" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I609" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>Medak</t>
+          <t>Mancherial</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
@@ -22978,35 +22978,35 @@
         </is>
       </c>
       <c r="D610" t="n">
-        <v>23.2</v>
+        <v>28</v>
       </c>
       <c r="E610" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="F610" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G610" t="n">
-        <v>12.7</v>
+        <v>14.8</v>
       </c>
       <c r="H610" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="I610" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>Medchal-Malkajgiri</t>
+          <t>Medak</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -23015,35 +23015,35 @@
         </is>
       </c>
       <c r="D611" t="n">
-        <v>22.4</v>
+        <v>27.8</v>
       </c>
       <c r="E611" t="n">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="F611" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="G611" t="n">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="H611" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="I611" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>Mulugu</t>
+          <t>Medchal-Malkajgiri</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -23052,35 +23052,35 @@
         </is>
       </c>
       <c r="D612" t="n">
-        <v>23.9</v>
+        <v>26.2</v>
       </c>
       <c r="E612" t="n">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="F612" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="G612" t="n">
-        <v>22</v>
+        <v>20.2</v>
       </c>
       <c r="H612" t="n">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="I612" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>Nagarkurnool</t>
+          <t>Mulugu</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -23089,35 +23089,35 @@
         </is>
       </c>
       <c r="D613" t="n">
-        <v>22.9</v>
+        <v>25.9</v>
       </c>
       <c r="E613" t="n">
         <v>94</v>
       </c>
       <c r="F613" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G613" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="H613" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I613" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>Nalgonda</t>
+          <t>Nagarkurnool</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -23126,35 +23126,35 @@
         </is>
       </c>
       <c r="D614" t="n">
-        <v>24.7</v>
+        <v>28.1</v>
       </c>
       <c r="E614" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="F614" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G614" t="n">
-        <v>17.2</v>
+        <v>25.8</v>
       </c>
       <c r="H614" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I614" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>Narayanpet</t>
+          <t>Nalgonda</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -23163,35 +23163,35 @@
         </is>
       </c>
       <c r="D615" t="n">
-        <v>23.4</v>
+        <v>27.1</v>
       </c>
       <c r="E615" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F615" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G615" t="n">
-        <v>14.9</v>
+        <v>18.5</v>
       </c>
       <c r="H615" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I615" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>Nirmal</t>
+          <t>Narayanpet</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
@@ -23200,35 +23200,35 @@
         </is>
       </c>
       <c r="D616" t="n">
-        <v>24.1</v>
+        <v>29</v>
       </c>
       <c r="E616" t="n">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="F616" t="n">
         <v>0.1</v>
       </c>
       <c r="G616" t="n">
-        <v>15.9</v>
+        <v>24.4</v>
       </c>
       <c r="H616" t="n">
         <v>51</v>
       </c>
       <c r="I616" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Nizamabad</t>
+          <t>Nirmal</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -23237,35 +23237,35 @@
         </is>
       </c>
       <c r="D617" t="n">
-        <v>23.8</v>
+        <v>29.3</v>
       </c>
       <c r="E617" t="n">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="F617" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G617" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="H617" t="n">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="I617" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>Peddapalli</t>
+          <t>Nizamabad</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -23274,35 +23274,35 @@
         </is>
       </c>
       <c r="D618" t="n">
-        <v>24.3</v>
+        <v>28.1</v>
       </c>
       <c r="E618" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="F618" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G618" t="n">
-        <v>19.1</v>
+        <v>18</v>
       </c>
       <c r="H618" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I618" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>Rajanna Sircilla</t>
+          <t>Peddapalli</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
@@ -23311,35 +23311,35 @@
         </is>
       </c>
       <c r="D619" t="n">
-        <v>24.1</v>
+        <v>27.1</v>
       </c>
       <c r="E619" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F619" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G619" t="n">
-        <v>15.1</v>
+        <v>20.4</v>
       </c>
       <c r="H619" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I619" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>Rangareddy</t>
+          <t>Rajanna Sircilla</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -23348,35 +23348,35 @@
         </is>
       </c>
       <c r="D620" t="n">
-        <v>22.6</v>
+        <v>28</v>
       </c>
       <c r="E620" t="n">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="F620" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G620" t="n">
-        <v>19.6</v>
+        <v>18.3</v>
       </c>
       <c r="H620" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I620" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>Sangareddy</t>
+          <t>Rangareddy</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -23385,35 +23385,35 @@
         </is>
       </c>
       <c r="D621" t="n">
-        <v>23.3</v>
+        <v>28.2</v>
       </c>
       <c r="E621" t="n">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="F621" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G621" t="n">
-        <v>17.1</v>
+        <v>26.7</v>
       </c>
       <c r="H621" t="n">
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="I621" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>Siddipet</t>
+          <t>Sangareddy</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -23422,35 +23422,35 @@
         </is>
       </c>
       <c r="D622" t="n">
-        <v>23.2</v>
+        <v>28.9</v>
       </c>
       <c r="E622" t="n">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="F622" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G622" t="n">
-        <v>23</v>
+        <v>26.4</v>
       </c>
       <c r="H622" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I622" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>Suryapet</t>
+          <t>Siddipet</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -23459,35 +23459,35 @@
         </is>
       </c>
       <c r="D623" t="n">
-        <v>24.9</v>
+        <v>26.7</v>
       </c>
       <c r="E623" t="n">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F623" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G623" t="n">
-        <v>22.5</v>
+        <v>23.8</v>
       </c>
       <c r="H623" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I623" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>Vikarabad</t>
+          <t>Suryapet</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
@@ -23496,35 +23496,35 @@
         </is>
       </c>
       <c r="D624" t="n">
-        <v>21.9</v>
+        <v>26.5</v>
       </c>
       <c r="E624" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F624" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G624" t="n">
-        <v>16.3</v>
+        <v>21.1</v>
       </c>
       <c r="H624" t="n">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="I624" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>Wanaparthy</t>
+          <t>Vikarabad</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
@@ -23533,35 +23533,35 @@
         </is>
       </c>
       <c r="D625" t="n">
-        <v>23.8</v>
+        <v>28.1</v>
       </c>
       <c r="E625" t="n">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="F625" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G625" t="n">
-        <v>14.8</v>
+        <v>25.5</v>
       </c>
       <c r="H625" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I625" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>Warangal</t>
+          <t>Wanaparthy</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -23570,35 +23570,35 @@
         </is>
       </c>
       <c r="D626" t="n">
-        <v>24.2</v>
+        <v>29.6</v>
       </c>
       <c r="E626" t="n">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="F626" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G626" t="n">
-        <v>21.9</v>
+        <v>26.1</v>
       </c>
       <c r="H626" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I626" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>Yadadri Bhuvanagiri</t>
+          <t>Warangal</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -23607,35 +23607,35 @@
         </is>
       </c>
       <c r="D627" t="n">
-        <v>23.4</v>
+        <v>25.6</v>
       </c>
       <c r="E627" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F627" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="G627" t="n">
-        <v>18.7</v>
+        <v>19.4</v>
       </c>
       <c r="H627" t="n">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="I627" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>Adilabad</t>
+          <t>Yadadri Bhuvanagiri</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -23644,2428 +23644,23 @@
         </is>
       </c>
       <c r="D628" t="n">
-        <v>24.2</v>
+        <v>25.8</v>
       </c>
       <c r="E628" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F628" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G628" t="n">
-        <v>13.2</v>
+        <v>20.1</v>
       </c>
       <c r="H628" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I628" t="inlineStr">
         <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="629">
-      <c r="A629" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B629" t="inlineStr">
-        <is>
-          <t>Bhadradri Kothagudem</t>
-        </is>
-      </c>
-      <c r="C629" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D629" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E629" t="n">
-        <v>96</v>
-      </c>
-      <c r="F629" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G629" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="H629" t="n">
-        <v>80</v>
-      </c>
-      <c r="I629" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="630">
-      <c r="A630" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B630" t="inlineStr">
-        <is>
-          <t>Hanumakonda</t>
-        </is>
-      </c>
-      <c r="C630" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D630" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="E630" t="n">
-        <v>94</v>
-      </c>
-      <c r="F630" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G630" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="H630" t="n">
-        <v>80</v>
-      </c>
-      <c r="I630" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="631">
-      <c r="A631" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B631" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D631" t="n">
-        <v>23</v>
-      </c>
-      <c r="E631" t="n">
-        <v>92</v>
-      </c>
-      <c r="F631" t="n">
-        <v>0</v>
-      </c>
-      <c r="G631" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="H631" t="n">
-        <v>3</v>
-      </c>
-      <c r="I631" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="632">
-      <c r="A632" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B632" t="inlineStr">
-        <is>
-          <t>Jagtial</t>
-        </is>
-      </c>
-      <c r="C632" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D632" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E632" t="n">
-        <v>96</v>
-      </c>
-      <c r="F632" t="n">
-        <v>0</v>
-      </c>
-      <c r="G632" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="H632" t="n">
-        <v>3</v>
-      </c>
-      <c r="I632" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="633">
-      <c r="A633" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B633" t="inlineStr">
-        <is>
-          <t>Jangaon</t>
-        </is>
-      </c>
-      <c r="C633" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D633" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E633" t="n">
-        <v>92</v>
-      </c>
-      <c r="F633" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G633" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="H633" t="n">
-        <v>80</v>
-      </c>
-      <c r="I633" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="634">
-      <c r="A634" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B634" t="inlineStr">
-        <is>
-          <t>Jayashankar Bhupalpally</t>
-        </is>
-      </c>
-      <c r="C634" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D634" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E634" t="n">
-        <v>99</v>
-      </c>
-      <c r="F634" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G634" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="H634" t="n">
-        <v>95</v>
-      </c>
-      <c r="I634" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="635">
-      <c r="A635" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B635" t="inlineStr">
-        <is>
-          <t>Jogulamba Gadwal</t>
-        </is>
-      </c>
-      <c r="C635" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D635" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="E635" t="n">
-        <v>82</v>
-      </c>
-      <c r="F635" t="n">
-        <v>0</v>
-      </c>
-      <c r="G635" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="H635" t="n">
-        <v>3</v>
-      </c>
-      <c r="I635" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="636">
-      <c r="A636" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B636" t="inlineStr">
-        <is>
-          <t>Kamareddy</t>
-        </is>
-      </c>
-      <c r="C636" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D636" t="n">
-        <v>23</v>
-      </c>
-      <c r="E636" t="n">
-        <v>95</v>
-      </c>
-      <c r="F636" t="n">
-        <v>0</v>
-      </c>
-      <c r="G636" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="H636" t="n">
-        <v>3</v>
-      </c>
-      <c r="I636" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="637">
-      <c r="A637" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B637" t="inlineStr">
-        <is>
-          <t>Karimnagar</t>
-        </is>
-      </c>
-      <c r="C637" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D637" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="E637" t="n">
-        <v>94</v>
-      </c>
-      <c r="F637" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G637" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="H637" t="n">
-        <v>53</v>
-      </c>
-      <c r="I637" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="638">
-      <c r="A638" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B638" t="inlineStr">
-        <is>
-          <t>Khammam</t>
-        </is>
-      </c>
-      <c r="C638" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D638" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E638" t="n">
-        <v>94</v>
-      </c>
-      <c r="F638" t="n">
-        <v>1</v>
-      </c>
-      <c r="G638" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="H638" t="n">
-        <v>81</v>
-      </c>
-      <c r="I638" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="639">
-      <c r="A639" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B639" t="inlineStr">
-        <is>
-          <t>Kumuram Bheem Asifabad</t>
-        </is>
-      </c>
-      <c r="C639" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D639" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="E639" t="n">
-        <v>94</v>
-      </c>
-      <c r="F639" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G639" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="H639" t="n">
-        <v>53</v>
-      </c>
-      <c r="I639" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="640">
-      <c r="A640" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B640" t="inlineStr">
-        <is>
-          <t>Mahabubabad</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D640" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="E640" t="n">
-        <v>95</v>
-      </c>
-      <c r="F640" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G640" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="H640" t="n">
-        <v>81</v>
-      </c>
-      <c r="I640" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="641">
-      <c r="A641" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B641" t="inlineStr">
-        <is>
-          <t>Mahbubnagar</t>
-        </is>
-      </c>
-      <c r="C641" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D641" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="E641" t="n">
-        <v>94</v>
-      </c>
-      <c r="F641" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G641" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="H641" t="n">
-        <v>51</v>
-      </c>
-      <c r="I641" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="642">
-      <c r="A642" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B642" t="inlineStr">
-        <is>
-          <t>Mancherial</t>
-        </is>
-      </c>
-      <c r="C642" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D642" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E642" t="n">
-        <v>96</v>
-      </c>
-      <c r="F642" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G642" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="H642" t="n">
-        <v>55</v>
-      </c>
-      <c r="I642" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="643">
-      <c r="A643" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B643" t="inlineStr">
-        <is>
-          <t>Medak</t>
-        </is>
-      </c>
-      <c r="C643" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D643" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="E643" t="n">
-        <v>96</v>
-      </c>
-      <c r="F643" t="n">
-        <v>0</v>
-      </c>
-      <c r="G643" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="H643" t="n">
-        <v>3</v>
-      </c>
-      <c r="I643" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="644">
-      <c r="A644" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B644" t="inlineStr">
-        <is>
-          <t>Medchal-Malkajgiri</t>
-        </is>
-      </c>
-      <c r="C644" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D644" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="E644" t="n">
-        <v>95</v>
-      </c>
-      <c r="F644" t="n">
-        <v>0</v>
-      </c>
-      <c r="G644" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="H644" t="n">
-        <v>3</v>
-      </c>
-      <c r="I644" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="645">
-      <c r="A645" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B645" t="inlineStr">
-        <is>
-          <t>Mulugu</t>
-        </is>
-      </c>
-      <c r="C645" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D645" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="E645" t="n">
-        <v>99</v>
-      </c>
-      <c r="F645" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G645" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="H645" t="n">
-        <v>95</v>
-      </c>
-      <c r="I645" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="646">
-      <c r="A646" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B646" t="inlineStr">
-        <is>
-          <t>Nagarkurnool</t>
-        </is>
-      </c>
-      <c r="C646" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D646" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="E646" t="n">
-        <v>94</v>
-      </c>
-      <c r="F646" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G646" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="H646" t="n">
-        <v>53</v>
-      </c>
-      <c r="I646" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="647">
-      <c r="A647" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B647" t="inlineStr">
-        <is>
-          <t>Nalgonda</t>
-        </is>
-      </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D647" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E647" t="n">
-        <v>91</v>
-      </c>
-      <c r="F647" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G647" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="H647" t="n">
-        <v>80</v>
-      </c>
-      <c r="I647" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="648">
-      <c r="A648" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B648" t="inlineStr">
-        <is>
-          <t>Narayanpet</t>
-        </is>
-      </c>
-      <c r="C648" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D648" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E648" t="n">
-        <v>88</v>
-      </c>
-      <c r="F648" t="n">
-        <v>0</v>
-      </c>
-      <c r="G648" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="H648" t="n">
-        <v>3</v>
-      </c>
-      <c r="I648" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="649">
-      <c r="A649" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B649" t="inlineStr">
-        <is>
-          <t>Nirmal</t>
-        </is>
-      </c>
-      <c r="C649" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D649" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="E649" t="n">
-        <v>94</v>
-      </c>
-      <c r="F649" t="n">
-        <v>0</v>
-      </c>
-      <c r="G649" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="H649" t="n">
-        <v>3</v>
-      </c>
-      <c r="I649" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="650">
-      <c r="A650" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B650" t="inlineStr">
-        <is>
-          <t>Nizamabad</t>
-        </is>
-      </c>
-      <c r="C650" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D650" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="E650" t="n">
-        <v>96</v>
-      </c>
-      <c r="F650" t="n">
-        <v>0</v>
-      </c>
-      <c r="G650" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="H650" t="n">
-        <v>3</v>
-      </c>
-      <c r="I650" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="651">
-      <c r="A651" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B651" t="inlineStr">
-        <is>
-          <t>Peddapalli</t>
-        </is>
-      </c>
-      <c r="C651" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D651" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E651" t="n">
-        <v>96</v>
-      </c>
-      <c r="F651" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G651" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="H651" t="n">
-        <v>80</v>
-      </c>
-      <c r="I651" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="652">
-      <c r="A652" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B652" t="inlineStr">
-        <is>
-          <t>Rajanna Sircilla</t>
-        </is>
-      </c>
-      <c r="C652" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D652" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E652" t="n">
-        <v>94</v>
-      </c>
-      <c r="F652" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G652" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="H652" t="n">
-        <v>51</v>
-      </c>
-      <c r="I652" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="653">
-      <c r="A653" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B653" t="inlineStr">
-        <is>
-          <t>Rangareddy</t>
-        </is>
-      </c>
-      <c r="C653" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D653" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="E653" t="n">
-        <v>95</v>
-      </c>
-      <c r="F653" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G653" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="H653" t="n">
-        <v>51</v>
-      </c>
-      <c r="I653" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="654">
-      <c r="A654" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B654" t="inlineStr">
-        <is>
-          <t>Sangareddy</t>
-        </is>
-      </c>
-      <c r="C654" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D654" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="E654" t="n">
-        <v>92</v>
-      </c>
-      <c r="F654" t="n">
-        <v>0</v>
-      </c>
-      <c r="G654" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="H654" t="n">
-        <v>3</v>
-      </c>
-      <c r="I654" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="655">
-      <c r="A655" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B655" t="inlineStr">
-        <is>
-          <t>Siddipet</t>
-        </is>
-      </c>
-      <c r="C655" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D655" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="E655" t="n">
-        <v>96</v>
-      </c>
-      <c r="F655" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G655" t="n">
-        <v>20.3</v>
-      </c>
-      <c r="H655" t="n">
-        <v>80</v>
-      </c>
-      <c r="I655" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="656">
-      <c r="A656" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B656" t="inlineStr">
-        <is>
-          <t>Suryapet</t>
-        </is>
-      </c>
-      <c r="C656" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D656" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E656" t="n">
-        <v>92</v>
-      </c>
-      <c r="F656" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G656" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="H656" t="n">
-        <v>80</v>
-      </c>
-      <c r="I656" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="657">
-      <c r="A657" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B657" t="inlineStr">
-        <is>
-          <t>Vikarabad</t>
-        </is>
-      </c>
-      <c r="C657" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D657" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="E657" t="n">
-        <v>96</v>
-      </c>
-      <c r="F657" t="n">
-        <v>0</v>
-      </c>
-      <c r="G657" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="H657" t="n">
-        <v>3</v>
-      </c>
-      <c r="I657" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="658">
-      <c r="A658" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B658" t="inlineStr">
-        <is>
-          <t>Wanaparthy</t>
-        </is>
-      </c>
-      <c r="C658" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D658" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="E658" t="n">
-        <v>90</v>
-      </c>
-      <c r="F658" t="n">
-        <v>0</v>
-      </c>
-      <c r="G658" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="H658" t="n">
-        <v>3</v>
-      </c>
-      <c r="I658" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="659">
-      <c r="A659" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B659" t="inlineStr">
-        <is>
-          <t>Warangal</t>
-        </is>
-      </c>
-      <c r="C659" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D659" t="n">
-        <v>24</v>
-      </c>
-      <c r="E659" t="n">
-        <v>95</v>
-      </c>
-      <c r="F659" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G659" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="H659" t="n">
-        <v>80</v>
-      </c>
-      <c r="I659" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B660" t="inlineStr">
-        <is>
-          <t>Yadadri Bhuvanagiri</t>
-        </is>
-      </c>
-      <c r="C660" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D660" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="E660" t="n">
-        <v>92</v>
-      </c>
-      <c r="F660" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G660" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="H660" t="n">
-        <v>51</v>
-      </c>
-      <c r="I660" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="661">
-      <c r="A661" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B661" t="inlineStr">
-        <is>
-          <t>Adilabad</t>
-        </is>
-      </c>
-      <c r="C661" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D661" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E661" t="n">
-        <v>94</v>
-      </c>
-      <c r="F661" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G661" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="H661" t="n">
-        <v>80</v>
-      </c>
-      <c r="I661" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B662" t="inlineStr">
-        <is>
-          <t>Bhadradri Kothagudem</t>
-        </is>
-      </c>
-      <c r="C662" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D662" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="E662" t="n">
-        <v>96</v>
-      </c>
-      <c r="F662" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G662" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="H662" t="n">
-        <v>55</v>
-      </c>
-      <c r="I662" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B663" t="inlineStr">
-        <is>
-          <t>Hanumakonda</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D663" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E663" t="n">
-        <v>95</v>
-      </c>
-      <c r="F663" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G663" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="H663" t="n">
-        <v>81</v>
-      </c>
-      <c r="I663" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="664">
-      <c r="A664" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B664" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="C664" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D664" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="E664" t="n">
-        <v>90</v>
-      </c>
-      <c r="F664" t="n">
-        <v>0</v>
-      </c>
-      <c r="G664" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="H664" t="n">
-        <v>3</v>
-      </c>
-      <c r="I664" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="665">
-      <c r="A665" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B665" t="inlineStr">
-        <is>
-          <t>Jagtial</t>
-        </is>
-      </c>
-      <c r="C665" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D665" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="E665" t="n">
-        <v>96</v>
-      </c>
-      <c r="F665" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G665" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="H665" t="n">
-        <v>80</v>
-      </c>
-      <c r="I665" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="666">
-      <c r="A666" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B666" t="inlineStr">
-        <is>
-          <t>Jangaon</t>
-        </is>
-      </c>
-      <c r="C666" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D666" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="E666" t="n">
-        <v>91</v>
-      </c>
-      <c r="F666" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G666" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="H666" t="n">
-        <v>80</v>
-      </c>
-      <c r="I666" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="667">
-      <c r="A667" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B667" t="inlineStr">
-        <is>
-          <t>Jayashankar Bhupalpally</t>
-        </is>
-      </c>
-      <c r="C667" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D667" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E667" t="n">
-        <v>99</v>
-      </c>
-      <c r="F667" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G667" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="H667" t="n">
-        <v>53</v>
-      </c>
-      <c r="I667" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B668" t="inlineStr">
-        <is>
-          <t>Jogulamba Gadwal</t>
-        </is>
-      </c>
-      <c r="C668" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D668" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="E668" t="n">
-        <v>87</v>
-      </c>
-      <c r="F668" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G668" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="H668" t="n">
-        <v>53</v>
-      </c>
-      <c r="I668" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="669">
-      <c r="A669" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B669" t="inlineStr">
-        <is>
-          <t>Kamareddy</t>
-        </is>
-      </c>
-      <c r="C669" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D669" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="E669" t="n">
-        <v>92</v>
-      </c>
-      <c r="F669" t="n">
-        <v>0</v>
-      </c>
-      <c r="G669" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="H669" t="n">
-        <v>3</v>
-      </c>
-      <c r="I669" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="670">
-      <c r="A670" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B670" t="inlineStr">
-        <is>
-          <t>Karimnagar</t>
-        </is>
-      </c>
-      <c r="C670" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D670" t="n">
-        <v>24</v>
-      </c>
-      <c r="E670" t="n">
-        <v>94</v>
-      </c>
-      <c r="F670" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G670" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="H670" t="n">
-        <v>53</v>
-      </c>
-      <c r="I670" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="671">
-      <c r="A671" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B671" t="inlineStr">
-        <is>
-          <t>Khammam</t>
-        </is>
-      </c>
-      <c r="C671" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D671" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="E671" t="n">
-        <v>94</v>
-      </c>
-      <c r="F671" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G671" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="H671" t="n">
-        <v>80</v>
-      </c>
-      <c r="I671" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="672">
-      <c r="A672" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B672" t="inlineStr">
-        <is>
-          <t>Kumuram Bheem Asifabad</t>
-        </is>
-      </c>
-      <c r="C672" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D672" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="E672" t="n">
-        <v>95</v>
-      </c>
-      <c r="F672" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G672" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="H672" t="n">
-        <v>51</v>
-      </c>
-      <c r="I672" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="673">
-      <c r="A673" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B673" t="inlineStr">
-        <is>
-          <t>Mahabubabad</t>
-        </is>
-      </c>
-      <c r="C673" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D673" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="E673" t="n">
-        <v>95</v>
-      </c>
-      <c r="F673" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G673" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="H673" t="n">
-        <v>80</v>
-      </c>
-      <c r="I673" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="674">
-      <c r="A674" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B674" t="inlineStr">
-        <is>
-          <t>Mahbubnagar</t>
-        </is>
-      </c>
-      <c r="C674" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D674" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="E674" t="n">
-        <v>92</v>
-      </c>
-      <c r="F674" t="n">
-        <v>0</v>
-      </c>
-      <c r="G674" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="H674" t="n">
-        <v>3</v>
-      </c>
-      <c r="I674" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="675">
-      <c r="A675" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B675" t="inlineStr">
-        <is>
-          <t>Mancherial</t>
-        </is>
-      </c>
-      <c r="C675" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D675" t="n">
-        <v>25</v>
-      </c>
-      <c r="E675" t="n">
-        <v>95</v>
-      </c>
-      <c r="F675" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G675" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="H675" t="n">
-        <v>51</v>
-      </c>
-      <c r="I675" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="676">
-      <c r="A676" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B676" t="inlineStr">
-        <is>
-          <t>Medak</t>
-        </is>
-      </c>
-      <c r="C676" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D676" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="E676" t="n">
-        <v>93</v>
-      </c>
-      <c r="F676" t="n">
-        <v>0</v>
-      </c>
-      <c r="G676" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="H676" t="n">
-        <v>3</v>
-      </c>
-      <c r="I676" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="677">
-      <c r="A677" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B677" t="inlineStr">
-        <is>
-          <t>Medchal-Malkajgiri</t>
-        </is>
-      </c>
-      <c r="C677" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D677" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="E677" t="n">
-        <v>94</v>
-      </c>
-      <c r="F677" t="n">
-        <v>0</v>
-      </c>
-      <c r="G677" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="H677" t="n">
-        <v>3</v>
-      </c>
-      <c r="I677" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="678">
-      <c r="A678" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B678" t="inlineStr">
-        <is>
-          <t>Mulugu</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D678" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="E678" t="n">
-        <v>98</v>
-      </c>
-      <c r="F678" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G678" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="H678" t="n">
-        <v>53</v>
-      </c>
-      <c r="I678" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="679">
-      <c r="A679" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B679" t="inlineStr">
-        <is>
-          <t>Nagarkurnool</t>
-        </is>
-      </c>
-      <c r="C679" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D679" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="E679" t="n">
-        <v>93</v>
-      </c>
-      <c r="F679" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G679" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="H679" t="n">
-        <v>51</v>
-      </c>
-      <c r="I679" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="680">
-      <c r="A680" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B680" t="inlineStr">
-        <is>
-          <t>Nalgonda</t>
-        </is>
-      </c>
-      <c r="C680" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D680" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E680" t="n">
-        <v>90</v>
-      </c>
-      <c r="F680" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G680" t="n">
-        <v>20</v>
-      </c>
-      <c r="H680" t="n">
-        <v>80</v>
-      </c>
-      <c r="I680" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B681" t="inlineStr">
-        <is>
-          <t>Narayanpet</t>
-        </is>
-      </c>
-      <c r="C681" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D681" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E681" t="n">
-        <v>85</v>
-      </c>
-      <c r="F681" t="n">
-        <v>0</v>
-      </c>
-      <c r="G681" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="H681" t="n">
-        <v>3</v>
-      </c>
-      <c r="I681" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="682">
-      <c r="A682" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B682" t="inlineStr">
-        <is>
-          <t>Nirmal</t>
-        </is>
-      </c>
-      <c r="C682" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D682" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E682" t="n">
-        <v>90</v>
-      </c>
-      <c r="F682" t="n">
-        <v>0</v>
-      </c>
-      <c r="G682" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="H682" t="n">
-        <v>3</v>
-      </c>
-      <c r="I682" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="683">
-      <c r="A683" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B683" t="inlineStr">
-        <is>
-          <t>Nizamabad</t>
-        </is>
-      </c>
-      <c r="C683" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D683" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E683" t="n">
-        <v>91</v>
-      </c>
-      <c r="F683" t="n">
-        <v>0</v>
-      </c>
-      <c r="G683" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="H683" t="n">
-        <v>3</v>
-      </c>
-      <c r="I683" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="684">
-      <c r="A684" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B684" t="inlineStr">
-        <is>
-          <t>Peddapalli</t>
-        </is>
-      </c>
-      <c r="C684" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D684" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="E684" t="n">
-        <v>96</v>
-      </c>
-      <c r="F684" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G684" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="H684" t="n">
-        <v>55</v>
-      </c>
-      <c r="I684" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="685">
-      <c r="A685" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B685" t="inlineStr">
-        <is>
-          <t>Rajanna Sircilla</t>
-        </is>
-      </c>
-      <c r="C685" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D685" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E685" t="n">
-        <v>94</v>
-      </c>
-      <c r="F685" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G685" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="H685" t="n">
-        <v>53</v>
-      </c>
-      <c r="I685" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B686" t="inlineStr">
-        <is>
-          <t>Rangareddy</t>
-        </is>
-      </c>
-      <c r="C686" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D686" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="E686" t="n">
-        <v>92</v>
-      </c>
-      <c r="F686" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G686" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="H686" t="n">
-        <v>51</v>
-      </c>
-      <c r="I686" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B687" t="inlineStr">
-        <is>
-          <t>Sangareddy</t>
-        </is>
-      </c>
-      <c r="C687" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D687" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E687" t="n">
-        <v>87</v>
-      </c>
-      <c r="F687" t="n">
-        <v>0</v>
-      </c>
-      <c r="G687" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="H687" t="n">
-        <v>3</v>
-      </c>
-      <c r="I687" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B688" t="inlineStr">
-        <is>
-          <t>Siddipet</t>
-        </is>
-      </c>
-      <c r="C688" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D688" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="E688" t="n">
-        <v>94</v>
-      </c>
-      <c r="F688" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G688" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="H688" t="n">
-        <v>55</v>
-      </c>
-      <c r="I688" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B689" t="inlineStr">
-        <is>
-          <t>Suryapet</t>
-        </is>
-      </c>
-      <c r="C689" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D689" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E689" t="n">
-        <v>91</v>
-      </c>
-      <c r="F689" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G689" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="H689" t="n">
-        <v>53</v>
-      </c>
-      <c r="I689" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B690" t="inlineStr">
-        <is>
-          <t>Vikarabad</t>
-        </is>
-      </c>
-      <c r="C690" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D690" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="E690" t="n">
-        <v>93</v>
-      </c>
-      <c r="F690" t="n">
-        <v>0</v>
-      </c>
-      <c r="G690" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="H690" t="n">
-        <v>3</v>
-      </c>
-      <c r="I690" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B691" t="inlineStr">
-        <is>
-          <t>Wanaparthy</t>
-        </is>
-      </c>
-      <c r="C691" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D691" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="E691" t="n">
-        <v>90</v>
-      </c>
-      <c r="F691" t="n">
-        <v>0</v>
-      </c>
-      <c r="G691" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="H691" t="n">
-        <v>3</v>
-      </c>
-      <c r="I691" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="692">
-      <c r="A692" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B692" t="inlineStr">
-        <is>
-          <t>Warangal</t>
-        </is>
-      </c>
-      <c r="C692" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D692" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="E692" t="n">
-        <v>96</v>
-      </c>
-      <c r="F692" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G692" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="H692" t="n">
-        <v>81</v>
-      </c>
-      <c r="I692" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="693">
-      <c r="A693" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B693" t="inlineStr">
-        <is>
-          <t>Yadadri Bhuvanagiri</t>
-        </is>
-      </c>
-      <c r="C693" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D693" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="E693" t="n">
-        <v>91</v>
-      </c>
-      <c r="F693" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G693" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="H693" t="n">
-        <v>53</v>
-      </c>
-      <c r="I693" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
@@ -26080,7 +23675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27298,7 +24893,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -27310,29 +24905,29 @@
         <v>33</v>
       </c>
       <c r="D21" t="n">
-        <v>23.9</v>
+        <v>27.4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Khammam</t>
+          <t>Jogulamba Gadwal</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>25.7</v>
+        <v>30.3</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Vikarabad</t>
+          <t>Bhadradri Kothagudem</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>21.9</v>
+        <v>25.1</v>
       </c>
       <c r="I21" t="n">
-        <v>94.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>8.699999999999999</v>
+        <v>2.5</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -27340,141 +24935,19 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Siddipet</t>
+          <t>Jangaon</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>23</v>
+        <v>26.7</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-09-24T00:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>33</v>
-      </c>
-      <c r="D22" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Jogulamba Gadwal</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Medchal-Malkajgiri</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="I22" t="n">
-        <v>93.90000000000001</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Khammam</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Jangaon</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>2026-09-24T04:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>33</v>
-      </c>
-      <c r="D23" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Mancherial</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>25</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Vikarabad</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="I23" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="J23" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Hanumakonda</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Jangaon</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>2026-09-24T06:30</t>
+          <t>2026-09-24T11:15</t>
         </is>
       </c>
     </row>
@@ -27541,19 +25014,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>27.6</v>
+        <v>28.3</v>
       </c>
       <c r="D2" t="n">
         <v>31.7</v>
       </c>
       <c r="E2" t="n">
-        <v>23.9</v>
+        <v>24.9</v>
       </c>
       <c r="F2" t="n">
-        <v>83.5</v>
+        <v>81.2</v>
       </c>
       <c r="G2" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="3">
@@ -27568,19 +25041,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.3</v>
+        <v>28.7</v>
       </c>
       <c r="D3" t="n">
         <v>34.1</v>
       </c>
       <c r="E3" t="n">
-        <v>24.2</v>
+        <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>82.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="4">
@@ -27595,19 +25068,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.4</v>
+        <v>29</v>
       </c>
       <c r="D4" t="n">
         <v>33.5</v>
       </c>
       <c r="E4" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="F4" t="n">
-        <v>76.90000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>2.2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5">
@@ -27622,19 +25095,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>28.7</v>
       </c>
       <c r="D5" t="n">
         <v>32.2</v>
       </c>
       <c r="E5" t="n">
-        <v>23</v>
+        <v>24.7</v>
       </c>
       <c r="F5" t="n">
-        <v>69.7</v>
+        <v>66.2</v>
       </c>
       <c r="G5" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -27649,19 +25122,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.5</v>
+        <v>28.1</v>
       </c>
       <c r="D6" t="n">
         <v>31.4</v>
       </c>
       <c r="E6" t="n">
-        <v>23.6</v>
+        <v>25.1</v>
       </c>
       <c r="F6" t="n">
-        <v>84.2</v>
+        <v>82.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -27676,19 +25149,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.7</v>
+        <v>28.3</v>
       </c>
       <c r="D7" t="n">
         <v>32</v>
       </c>
       <c r="E7" t="n">
-        <v>23.6</v>
+        <v>24.4</v>
       </c>
       <c r="F7" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
@@ -27703,19 +25176,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27.7</v>
+        <v>28.2</v>
       </c>
       <c r="D8" t="n">
         <v>33</v>
       </c>
       <c r="E8" t="n">
-        <v>23.9</v>
+        <v>24.4</v>
       </c>
       <c r="F8" t="n">
-        <v>84.09999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="G8" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9">
@@ -27730,7 +25203,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.2</v>
+        <v>28.8</v>
       </c>
       <c r="D9" t="n">
         <v>34.2</v>
@@ -27739,10 +25212,10 @@
         <v>23.9</v>
       </c>
       <c r="F9" t="n">
-        <v>71.90000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="G9" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -27757,7 +25230,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.2</v>
+        <v>26.7</v>
       </c>
       <c r="D10" t="n">
         <v>30.1</v>
@@ -27766,10 +25239,10 @@
         <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>82.8</v>
+        <v>80.7</v>
       </c>
       <c r="G10" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="11">
@@ -27784,19 +25257,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28</v>
+        <v>28.5</v>
       </c>
       <c r="D11" t="n">
         <v>32</v>
       </c>
       <c r="E11" t="n">
-        <v>24</v>
+        <v>25.8</v>
       </c>
       <c r="F11" t="n">
-        <v>81.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
@@ -27811,19 +25284,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.3</v>
+        <v>29.8</v>
       </c>
       <c r="D12" t="n">
         <v>35.2</v>
       </c>
       <c r="E12" t="n">
-        <v>24.7</v>
+        <v>25.5</v>
       </c>
       <c r="F12" t="n">
-        <v>76.2</v>
+        <v>74.3</v>
       </c>
       <c r="G12" t="n">
-        <v>2.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="13">
@@ -27838,19 +25311,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>28</v>
+        <v>28.6</v>
       </c>
       <c r="D13" t="n">
         <v>32.8</v>
       </c>
       <c r="E13" t="n">
-        <v>24.4</v>
+        <v>25.2</v>
       </c>
       <c r="F13" t="n">
-        <v>83.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="14">
@@ -27865,19 +25338,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>28.3</v>
+        <v>28.8</v>
       </c>
       <c r="D14" t="n">
         <v>33.3</v>
       </c>
       <c r="E14" t="n">
-        <v>24.1</v>
+        <v>24.9</v>
       </c>
       <c r="F14" t="n">
-        <v>80.7</v>
+        <v>78.2</v>
       </c>
       <c r="G14" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="15">
@@ -27892,19 +25365,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.5</v>
+        <v>27.2</v>
       </c>
       <c r="D15" t="n">
         <v>31.1</v>
       </c>
       <c r="E15" t="n">
-        <v>22.4</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>77.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="16">
@@ -27919,19 +25392,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28.5</v>
+        <v>29</v>
       </c>
       <c r="D16" t="n">
         <v>32.7</v>
       </c>
       <c r="E16" t="n">
-        <v>24.7</v>
+        <v>26</v>
       </c>
       <c r="F16" t="n">
-        <v>81.2</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17">
@@ -27946,19 +25419,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26.6</v>
+        <v>27.2</v>
       </c>
       <c r="D17" t="n">
         <v>30.4</v>
       </c>
       <c r="E17" t="n">
-        <v>22.8</v>
+        <v>24</v>
       </c>
       <c r="F17" t="n">
-        <v>82</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="18">
@@ -27973,19 +25446,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26.4</v>
+        <v>27.1</v>
       </c>
       <c r="D18" t="n">
         <v>31.1</v>
       </c>
       <c r="E18" t="n">
-        <v>22.3</v>
+        <v>23.7</v>
       </c>
       <c r="F18" t="n">
-        <v>78.2</v>
+        <v>75.3</v>
       </c>
       <c r="G18" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="19">
@@ -28000,19 +25473,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="D19" t="n">
         <v>32</v>
       </c>
       <c r="E19" t="n">
-        <v>23.5</v>
+        <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>84.09999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="20">
@@ -28027,19 +25500,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27.1</v>
+        <v>27.8</v>
       </c>
       <c r="D20" t="n">
         <v>32.2</v>
       </c>
       <c r="E20" t="n">
-        <v>22.9</v>
+        <v>23.4</v>
       </c>
       <c r="F20" t="n">
-        <v>75.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="21">
@@ -28054,19 +25527,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>29.7</v>
+        <v>30.4</v>
       </c>
       <c r="D21" t="n">
         <v>36.2</v>
       </c>
       <c r="E21" t="n">
-        <v>24.7</v>
+        <v>25.7</v>
       </c>
       <c r="F21" t="n">
-        <v>69</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>2.2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="22">
@@ -28081,7 +25554,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>26.8</v>
+        <v>27.4</v>
       </c>
       <c r="D22" t="n">
         <v>31.4</v>
@@ -28090,10 +25563,10 @@
         <v>22.5</v>
       </c>
       <c r="F22" t="n">
-        <v>75.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="23">
@@ -28108,19 +25581,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>27.5</v>
+        <v>28.2</v>
       </c>
       <c r="D23" t="n">
         <v>31.6</v>
       </c>
       <c r="E23" t="n">
-        <v>23.7</v>
+        <v>24.4</v>
       </c>
       <c r="F23" t="n">
-        <v>80.09999999999999</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="24">
@@ -28135,19 +25608,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.8</v>
+        <v>27.4</v>
       </c>
       <c r="D24" t="n">
         <v>30.6</v>
       </c>
       <c r="E24" t="n">
-        <v>23.5</v>
+        <v>23.9</v>
       </c>
       <c r="F24" t="n">
-        <v>83.09999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="25">
@@ -28162,19 +25635,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28</v>
+        <v>28.5</v>
       </c>
       <c r="D25" t="n">
         <v>32</v>
       </c>
       <c r="E25" t="n">
-        <v>24.1</v>
+        <v>25.4</v>
       </c>
       <c r="F25" t="n">
-        <v>83.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="G25" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="26">
@@ -28189,19 +25662,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.5</v>
+        <v>28.1</v>
       </c>
       <c r="D26" t="n">
         <v>31.2</v>
       </c>
       <c r="E26" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="F26" t="n">
-        <v>81.59999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="G26" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="27">
@@ -28216,19 +25689,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26.5</v>
+        <v>27.2</v>
       </c>
       <c r="D27" t="n">
         <v>30.8</v>
       </c>
       <c r="E27" t="n">
-        <v>22.5</v>
+        <v>22.9</v>
       </c>
       <c r="F27" t="n">
-        <v>75.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G27" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="28">
@@ -28243,19 +25716,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.4</v>
+        <v>28.1</v>
       </c>
       <c r="D28" t="n">
         <v>31.9</v>
       </c>
       <c r="E28" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="F28" t="n">
-        <v>74.2</v>
+        <v>71.2</v>
       </c>
       <c r="G28" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="29">
@@ -28270,19 +25743,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.6</v>
+        <v>27.2</v>
       </c>
       <c r="D29" t="n">
         <v>30.2</v>
       </c>
       <c r="E29" t="n">
-        <v>22.8</v>
+        <v>24.2</v>
       </c>
       <c r="F29" t="n">
-        <v>81.8</v>
+        <v>79.7</v>
       </c>
       <c r="G29" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="30">
@@ -28297,19 +25770,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>29.4</v>
+        <v>30</v>
       </c>
       <c r="D30" t="n">
         <v>34.5</v>
       </c>
       <c r="E30" t="n">
-        <v>24.7</v>
+        <v>25.4</v>
       </c>
       <c r="F30" t="n">
-        <v>72</v>
+        <v>69.8</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31">
@@ -28324,19 +25797,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>26.3</v>
+        <v>27</v>
       </c>
       <c r="D31" t="n">
         <v>30.5</v>
       </c>
       <c r="E31" t="n">
-        <v>21.9</v>
+        <v>22.6</v>
       </c>
       <c r="F31" t="n">
-        <v>76.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -28351,16 +25824,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27.7</v>
+        <v>28.3</v>
       </c>
       <c r="D32" t="n">
         <v>32.1</v>
       </c>
       <c r="E32" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="F32" t="n">
-        <v>73.40000000000001</v>
+        <v>70.2</v>
       </c>
       <c r="G32" t="n">
         <v>3.3</v>
@@ -28378,19 +25851,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>28.6</v>
+        <v>29.2</v>
       </c>
       <c r="D33" t="n">
         <v>34.4</v>
       </c>
       <c r="E33" t="n">
-        <v>23.7</v>
+        <v>24.7</v>
       </c>
       <c r="F33" t="n">
-        <v>75.09999999999999</v>
+        <v>72.8</v>
       </c>
       <c r="G33" t="n">
-        <v>2.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="34">
@@ -28405,19 +25878,19 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>27.4</v>
+        <v>28</v>
       </c>
       <c r="D34" t="n">
         <v>32</v>
       </c>
       <c r="E34" t="n">
-        <v>23.4</v>
+        <v>24.5</v>
       </c>
       <c r="F34" t="n">
-        <v>75.8</v>
+        <v>73.7</v>
       </c>
       <c r="G34" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update weather analytics outputs
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I694"/>
+  <dimension ref="A1:I661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23681,23 +23681,23 @@
         </is>
       </c>
       <c r="D629" t="n">
-        <v>30</v>
+        <v>25.7</v>
       </c>
       <c r="E629" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="F629" t="n">
         <v>0</v>
       </c>
       <c r="G629" t="n">
-        <v>20.5</v>
+        <v>19.2</v>
       </c>
       <c r="H629" t="n">
         <v>3</v>
       </c>
       <c r="I629" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23718,23 +23718,23 @@
         </is>
       </c>
       <c r="D630" t="n">
-        <v>26.9</v>
+        <v>25.1</v>
       </c>
       <c r="E630" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F630" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G630" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="H630" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I630" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23755,23 +23755,23 @@
         </is>
       </c>
       <c r="D631" t="n">
-        <v>27.3</v>
+        <v>25.4</v>
       </c>
       <c r="E631" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F631" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G631" t="n">
-        <v>21.5</v>
+        <v>19.2</v>
       </c>
       <c r="H631" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I631" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23792,23 +23792,23 @@
         </is>
       </c>
       <c r="D632" t="n">
-        <v>27.9</v>
+        <v>26.1</v>
       </c>
       <c r="E632" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F632" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G632" t="n">
-        <v>19.4</v>
+        <v>14.2</v>
       </c>
       <c r="H632" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I632" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23829,23 +23829,23 @@
         </is>
       </c>
       <c r="D633" t="n">
-        <v>29.3</v>
+        <v>25.4</v>
       </c>
       <c r="E633" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F633" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G633" t="n">
-        <v>19.6</v>
+        <v>17.8</v>
       </c>
       <c r="H633" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I633" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23866,23 +23866,23 @@
         </is>
       </c>
       <c r="D634" t="n">
-        <v>27.7</v>
+        <v>26.7</v>
       </c>
       <c r="E634" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F634" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G634" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
       <c r="H634" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="I634" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23903,23 +23903,23 @@
         </is>
       </c>
       <c r="D635" t="n">
-        <v>27.4</v>
+        <v>24.5</v>
       </c>
       <c r="E635" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="F635" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G635" t="n">
-        <v>20.9</v>
+        <v>17.9</v>
       </c>
       <c r="H635" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="I635" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23940,23 +23940,23 @@
         </is>
       </c>
       <c r="D636" t="n">
-        <v>31.4</v>
+        <v>26.9</v>
       </c>
       <c r="E636" t="n">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="F636" t="n">
         <v>0</v>
       </c>
       <c r="G636" t="n">
-        <v>26.7</v>
+        <v>22.3</v>
       </c>
       <c r="H636" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I636" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -23977,23 +23977,23 @@
         </is>
       </c>
       <c r="D637" t="n">
-        <v>28.2</v>
+        <v>25.3</v>
       </c>
       <c r="E637" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F637" t="n">
         <v>0</v>
       </c>
       <c r="G637" t="n">
-        <v>23.5</v>
+        <v>21.1</v>
       </c>
       <c r="H637" t="n">
         <v>3</v>
       </c>
       <c r="I637" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24014,23 +24014,23 @@
         </is>
       </c>
       <c r="D638" t="n">
-        <v>29.1</v>
+        <v>26</v>
       </c>
       <c r="E638" t="n">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F638" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G638" t="n">
-        <v>20.4</v>
+        <v>16.6</v>
       </c>
       <c r="H638" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="I638" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24051,23 +24051,23 @@
         </is>
       </c>
       <c r="D639" t="n">
-        <v>26.4</v>
+        <v>25.4</v>
       </c>
       <c r="E639" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F639" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G639" t="n">
-        <v>19.4</v>
+        <v>16.2</v>
       </c>
       <c r="H639" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I639" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24088,23 +24088,23 @@
         </is>
       </c>
       <c r="D640" t="n">
-        <v>26.9</v>
+        <v>24.8</v>
       </c>
       <c r="E640" t="n">
         <v>93</v>
       </c>
       <c r="F640" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G640" t="n">
-        <v>17.6</v>
+        <v>18.6</v>
       </c>
       <c r="H640" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="I640" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24125,23 +24125,23 @@
         </is>
       </c>
       <c r="D641" t="n">
-        <v>26.3</v>
+        <v>25.3</v>
       </c>
       <c r="E641" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F641" t="n">
         <v>0.1</v>
       </c>
       <c r="G641" t="n">
-        <v>21</v>
+        <v>15.4</v>
       </c>
       <c r="H641" t="n">
         <v>51</v>
       </c>
       <c r="I641" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24162,23 +24162,23 @@
         </is>
       </c>
       <c r="D642" t="n">
-        <v>29.8</v>
+        <v>25.8</v>
       </c>
       <c r="E642" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F642" t="n">
         <v>0</v>
       </c>
       <c r="G642" t="n">
-        <v>24.5</v>
+        <v>17</v>
       </c>
       <c r="H642" t="n">
         <v>3</v>
       </c>
       <c r="I642" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24199,23 +24199,23 @@
         </is>
       </c>
       <c r="D643" t="n">
-        <v>29.5</v>
+        <v>25</v>
       </c>
       <c r="E643" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="F643" t="n">
-        <v>2.1</v>
+        <v>0.1</v>
       </c>
       <c r="G643" t="n">
-        <v>16.6</v>
+        <v>15.6</v>
       </c>
       <c r="H643" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="I643" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24236,23 +24236,23 @@
         </is>
       </c>
       <c r="D644" t="n">
-        <v>28.1</v>
+        <v>24.3</v>
       </c>
       <c r="E644" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F644" t="n">
         <v>0</v>
       </c>
       <c r="G644" t="n">
-        <v>23.1</v>
+        <v>11.7</v>
       </c>
       <c r="H644" t="n">
         <v>3</v>
       </c>
       <c r="I644" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24273,23 +24273,23 @@
         </is>
       </c>
       <c r="D645" t="n">
-        <v>27.3</v>
+        <v>25.3</v>
       </c>
       <c r="E645" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F645" t="n">
         <v>0</v>
       </c>
       <c r="G645" t="n">
-        <v>22.4</v>
+        <v>17.5</v>
       </c>
       <c r="H645" t="n">
         <v>3</v>
       </c>
       <c r="I645" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24310,23 +24310,23 @@
         </is>
       </c>
       <c r="D646" t="n">
-        <v>27.1</v>
+        <v>24.4</v>
       </c>
       <c r="E646" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F646" t="n">
         <v>0.1</v>
       </c>
       <c r="G646" t="n">
-        <v>20.7</v>
+        <v>19.6</v>
       </c>
       <c r="H646" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="I646" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24347,23 +24347,23 @@
         </is>
       </c>
       <c r="D647" t="n">
-        <v>29</v>
+        <v>25.3</v>
       </c>
       <c r="E647" t="n">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F647" t="n">
         <v>0</v>
       </c>
       <c r="G647" t="n">
-        <v>25.6</v>
+        <v>20.2</v>
       </c>
       <c r="H647" t="n">
         <v>3</v>
       </c>
       <c r="I647" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24384,23 +24384,23 @@
         </is>
       </c>
       <c r="D648" t="n">
-        <v>29</v>
+        <v>27.9</v>
       </c>
       <c r="E648" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F648" t="n">
         <v>0</v>
       </c>
       <c r="G648" t="n">
-        <v>19.1</v>
+        <v>14.6</v>
       </c>
       <c r="H648" t="n">
         <v>3</v>
       </c>
       <c r="I648" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24421,7 +24421,7 @@
         </is>
       </c>
       <c r="D649" t="n">
-        <v>30.1</v>
+        <v>26.1</v>
       </c>
       <c r="E649" t="n">
         <v>63</v>
@@ -24430,14 +24430,14 @@
         <v>0</v>
       </c>
       <c r="G649" t="n">
-        <v>23.6</v>
+        <v>16.6</v>
       </c>
       <c r="H649" t="n">
         <v>3</v>
       </c>
       <c r="I649" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24458,23 +24458,23 @@
         </is>
       </c>
       <c r="D650" t="n">
-        <v>30.6</v>
+        <v>25.9</v>
       </c>
       <c r="E650" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="F650" t="n">
         <v>0</v>
       </c>
       <c r="G650" t="n">
-        <v>20</v>
+        <v>18.9</v>
       </c>
       <c r="H650" t="n">
         <v>3</v>
       </c>
       <c r="I650" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24495,23 +24495,23 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>29.5</v>
+        <v>25.6</v>
       </c>
       <c r="E651" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F651" t="n">
         <v>0</v>
       </c>
       <c r="G651" t="n">
-        <v>19.7</v>
+        <v>15.3</v>
       </c>
       <c r="H651" t="n">
         <v>3</v>
       </c>
       <c r="I651" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24532,23 +24532,23 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="E652" t="n">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="F652" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G652" t="n">
-        <v>20.6</v>
+        <v>21.6</v>
       </c>
       <c r="H652" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24569,23 +24569,23 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>29.6</v>
+        <v>26.3</v>
       </c>
       <c r="E653" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F653" t="n">
         <v>0</v>
       </c>
       <c r="G653" t="n">
-        <v>19.7</v>
+        <v>20.1</v>
       </c>
       <c r="H653" t="n">
         <v>3</v>
       </c>
       <c r="I653" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24606,23 +24606,23 @@
         </is>
       </c>
       <c r="D654" t="n">
-        <v>28.4</v>
+        <v>25.7</v>
       </c>
       <c r="E654" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F654" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G654" t="n">
-        <v>25.6</v>
+        <v>20.5</v>
       </c>
       <c r="H654" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="I654" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24643,23 +24643,23 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>29.4</v>
+        <v>26.8</v>
       </c>
       <c r="E655" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F655" t="n">
         <v>0</v>
       </c>
       <c r="G655" t="n">
-        <v>23.7</v>
+        <v>18.9</v>
       </c>
       <c r="H655" t="n">
         <v>3</v>
       </c>
       <c r="I655" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24680,23 +24680,23 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>28.5</v>
+        <v>25.6</v>
       </c>
       <c r="E656" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F656" t="n">
         <v>0</v>
       </c>
       <c r="G656" t="n">
-        <v>21.7</v>
+        <v>24.3</v>
       </c>
       <c r="H656" t="n">
         <v>3</v>
       </c>
       <c r="I656" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24717,23 +24717,23 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>27.3</v>
+        <v>24.8</v>
       </c>
       <c r="E657" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F657" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G657" t="n">
-        <v>17.8</v>
+        <v>14.7</v>
       </c>
       <c r="H657" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I657" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24754,23 +24754,23 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>29.3</v>
+        <v>25</v>
       </c>
       <c r="E658" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F658" t="n">
         <v>0</v>
       </c>
       <c r="G658" t="n">
-        <v>24.2</v>
+        <v>17.6</v>
       </c>
       <c r="H658" t="n">
         <v>3</v>
       </c>
       <c r="I658" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24791,23 +24791,23 @@
         </is>
       </c>
       <c r="D659" t="n">
-        <v>30.4</v>
+        <v>25.6</v>
       </c>
       <c r="E659" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="F659" t="n">
         <v>0</v>
       </c>
       <c r="G659" t="n">
-        <v>25.8</v>
+        <v>15.9</v>
       </c>
       <c r="H659" t="n">
         <v>3</v>
       </c>
       <c r="I659" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24828,23 +24828,23 @@
         </is>
       </c>
       <c r="D660" t="n">
-        <v>27.1</v>
+        <v>25.4</v>
       </c>
       <c r="E660" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F660" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G660" t="n">
-        <v>21.5</v>
+        <v>19.8</v>
       </c>
       <c r="H660" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="I660" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -24865,1244 +24865,23 @@
         </is>
       </c>
       <c r="D661" t="n">
-        <v>27.8</v>
+        <v>26.4</v>
       </c>
       <c r="E661" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F661" t="n">
         <v>0</v>
       </c>
       <c r="G661" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="H661" t="n">
         <v>3</v>
       </c>
       <c r="I661" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B662" t="inlineStr">
-        <is>
-          <t>Adilabad</t>
-        </is>
-      </c>
-      <c r="C662" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D662" t="n">
-        <v>26</v>
-      </c>
-      <c r="E662" t="n">
-        <v>90</v>
-      </c>
-      <c r="F662" t="n">
-        <v>0</v>
-      </c>
-      <c r="G662" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="H662" t="n">
-        <v>3</v>
-      </c>
-      <c r="I662" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B663" t="inlineStr">
-        <is>
-          <t>Bhadradri Kothagudem</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D663" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="E663" t="n">
-        <v>95</v>
-      </c>
-      <c r="F663" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G663" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H663" t="n">
-        <v>80</v>
-      </c>
-      <c r="I663" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="664">
-      <c r="A664" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B664" t="inlineStr">
-        <is>
-          <t>Hanumakonda</t>
-        </is>
-      </c>
-      <c r="C664" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D664" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="E664" t="n">
-        <v>90</v>
-      </c>
-      <c r="F664" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G664" t="n">
-        <v>17</v>
-      </c>
-      <c r="H664" t="n">
-        <v>51</v>
-      </c>
-      <c r="I664" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="665">
-      <c r="A665" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B665" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="C665" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D665" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="E665" t="n">
-        <v>77</v>
-      </c>
-      <c r="F665" t="n">
-        <v>0</v>
-      </c>
-      <c r="G665" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="H665" t="n">
-        <v>3</v>
-      </c>
-      <c r="I665" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="666">
-      <c r="A666" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B666" t="inlineStr">
-        <is>
-          <t>Jagtial</t>
-        </is>
-      </c>
-      <c r="C666" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D666" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="E666" t="n">
-        <v>92</v>
-      </c>
-      <c r="F666" t="n">
-        <v>0</v>
-      </c>
-      <c r="G666" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="H666" t="n">
-        <v>3</v>
-      </c>
-      <c r="I666" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="667">
-      <c r="A667" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B667" t="inlineStr">
-        <is>
-          <t>Jangaon</t>
-        </is>
-      </c>
-      <c r="C667" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D667" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="E667" t="n">
-        <v>90</v>
-      </c>
-      <c r="F667" t="n">
-        <v>0</v>
-      </c>
-      <c r="G667" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="H667" t="n">
-        <v>3</v>
-      </c>
-      <c r="I667" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B668" t="inlineStr">
-        <is>
-          <t>Jayashankar Bhupalpally</t>
-        </is>
-      </c>
-      <c r="C668" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D668" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="E668" t="n">
-        <v>91</v>
-      </c>
-      <c r="F668" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G668" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="H668" t="n">
-        <v>51</v>
-      </c>
-      <c r="I668" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="669">
-      <c r="A669" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B669" t="inlineStr">
-        <is>
-          <t>Jogulamba Gadwal</t>
-        </is>
-      </c>
-      <c r="C669" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D669" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="E669" t="n">
-        <v>64</v>
-      </c>
-      <c r="F669" t="n">
-        <v>0</v>
-      </c>
-      <c r="G669" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="H669" t="n">
-        <v>3</v>
-      </c>
-      <c r="I669" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="670">
-      <c r="A670" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B670" t="inlineStr">
-        <is>
-          <t>Kamareddy</t>
-        </is>
-      </c>
-      <c r="C670" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D670" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="E670" t="n">
-        <v>93</v>
-      </c>
-      <c r="F670" t="n">
-        <v>0</v>
-      </c>
-      <c r="G670" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="H670" t="n">
-        <v>3</v>
-      </c>
-      <c r="I670" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="671">
-      <c r="A671" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B671" t="inlineStr">
-        <is>
-          <t>Karimnagar</t>
-        </is>
-      </c>
-      <c r="C671" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D671" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="E671" t="n">
-        <v>86</v>
-      </c>
-      <c r="F671" t="n">
-        <v>0</v>
-      </c>
-      <c r="G671" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="H671" t="n">
-        <v>3</v>
-      </c>
-      <c r="I671" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="672">
-      <c r="A672" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B672" t="inlineStr">
-        <is>
-          <t>Khammam</t>
-        </is>
-      </c>
-      <c r="C672" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D672" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="E672" t="n">
-        <v>83</v>
-      </c>
-      <c r="F672" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G672" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="H672" t="n">
-        <v>51</v>
-      </c>
-      <c r="I672" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="673">
-      <c r="A673" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B673" t="inlineStr">
-        <is>
-          <t>Kumuram Bheem Asifabad</t>
-        </is>
-      </c>
-      <c r="C673" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D673" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="E673" t="n">
-        <v>89</v>
-      </c>
-      <c r="F673" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G673" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="H673" t="n">
-        <v>51</v>
-      </c>
-      <c r="I673" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="674">
-      <c r="A674" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B674" t="inlineStr">
-        <is>
-          <t>Mahabubabad</t>
-        </is>
-      </c>
-      <c r="C674" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D674" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="E674" t="n">
-        <v>89</v>
-      </c>
-      <c r="F674" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G674" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H674" t="n">
-        <v>55</v>
-      </c>
-      <c r="I674" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="675">
-      <c r="A675" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B675" t="inlineStr">
-        <is>
-          <t>Mahbubnagar</t>
-        </is>
-      </c>
-      <c r="C675" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D675" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="E675" t="n">
-        <v>82</v>
-      </c>
-      <c r="F675" t="n">
-        <v>0</v>
-      </c>
-      <c r="G675" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="H675" t="n">
-        <v>3</v>
-      </c>
-      <c r="I675" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="676">
-      <c r="A676" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B676" t="inlineStr">
-        <is>
-          <t>Mancherial</t>
-        </is>
-      </c>
-      <c r="C676" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D676" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="E676" t="n">
-        <v>89</v>
-      </c>
-      <c r="F676" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G676" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="H676" t="n">
-        <v>53</v>
-      </c>
-      <c r="I676" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="677">
-      <c r="A677" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B677" t="inlineStr">
-        <is>
-          <t>Medak</t>
-        </is>
-      </c>
-      <c r="C677" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D677" t="n">
-        <v>25.1</v>
-      </c>
-      <c r="E677" t="n">
-        <v>92</v>
-      </c>
-      <c r="F677" t="n">
-        <v>0</v>
-      </c>
-      <c r="G677" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="H677" t="n">
-        <v>3</v>
-      </c>
-      <c r="I677" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="678">
-      <c r="A678" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B678" t="inlineStr">
-        <is>
-          <t>Medchal-Malkajgiri</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D678" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="E678" t="n">
-        <v>86</v>
-      </c>
-      <c r="F678" t="n">
-        <v>0</v>
-      </c>
-      <c r="G678" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="H678" t="n">
-        <v>3</v>
-      </c>
-      <c r="I678" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="679">
-      <c r="A679" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B679" t="inlineStr">
-        <is>
-          <t>Mulugu</t>
-        </is>
-      </c>
-      <c r="C679" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D679" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E679" t="n">
-        <v>95</v>
-      </c>
-      <c r="F679" t="n">
-        <v>0</v>
-      </c>
-      <c r="G679" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="H679" t="n">
-        <v>3</v>
-      </c>
-      <c r="I679" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="680">
-      <c r="A680" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B680" t="inlineStr">
-        <is>
-          <t>Nagarkurnool</t>
-        </is>
-      </c>
-      <c r="C680" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D680" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="E680" t="n">
-        <v>76</v>
-      </c>
-      <c r="F680" t="n">
-        <v>0</v>
-      </c>
-      <c r="G680" t="n">
-        <v>17</v>
-      </c>
-      <c r="H680" t="n">
-        <v>3</v>
-      </c>
-      <c r="I680" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B681" t="inlineStr">
-        <is>
-          <t>Nalgonda</t>
-        </is>
-      </c>
-      <c r="C681" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D681" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="E681" t="n">
-        <v>73</v>
-      </c>
-      <c r="F681" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G681" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="H681" t="n">
-        <v>51</v>
-      </c>
-      <c r="I681" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="682">
-      <c r="A682" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B682" t="inlineStr">
-        <is>
-          <t>Narayanpet</t>
-        </is>
-      </c>
-      <c r="C682" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D682" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="E682" t="n">
-        <v>73</v>
-      </c>
-      <c r="F682" t="n">
-        <v>0</v>
-      </c>
-      <c r="G682" t="n">
-        <v>14</v>
-      </c>
-      <c r="H682" t="n">
-        <v>3</v>
-      </c>
-      <c r="I682" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="683">
-      <c r="A683" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B683" t="inlineStr">
-        <is>
-          <t>Nirmal</t>
-        </is>
-      </c>
-      <c r="C683" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D683" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="E683" t="n">
-        <v>90</v>
-      </c>
-      <c r="F683" t="n">
-        <v>0</v>
-      </c>
-      <c r="G683" t="n">
-        <v>15</v>
-      </c>
-      <c r="H683" t="n">
-        <v>3</v>
-      </c>
-      <c r="I683" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="684">
-      <c r="A684" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B684" t="inlineStr">
-        <is>
-          <t>Nizamabad</t>
-        </is>
-      </c>
-      <c r="C684" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D684" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="E684" t="n">
-        <v>94</v>
-      </c>
-      <c r="F684" t="n">
-        <v>0</v>
-      </c>
-      <c r="G684" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="H684" t="n">
-        <v>3</v>
-      </c>
-      <c r="I684" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="685">
-      <c r="A685" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B685" t="inlineStr">
-        <is>
-          <t>Peddapalli</t>
-        </is>
-      </c>
-      <c r="C685" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D685" t="n">
-        <v>26</v>
-      </c>
-      <c r="E685" t="n">
-        <v>90</v>
-      </c>
-      <c r="F685" t="n">
-        <v>0</v>
-      </c>
-      <c r="G685" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="H685" t="n">
-        <v>3</v>
-      </c>
-      <c r="I685" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B686" t="inlineStr">
-        <is>
-          <t>Rajanna Sircilla</t>
-        </is>
-      </c>
-      <c r="C686" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D686" t="n">
-        <v>25</v>
-      </c>
-      <c r="E686" t="n">
-        <v>90</v>
-      </c>
-      <c r="F686" t="n">
-        <v>0</v>
-      </c>
-      <c r="G686" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="H686" t="n">
-        <v>3</v>
-      </c>
-      <c r="I686" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B687" t="inlineStr">
-        <is>
-          <t>Rangareddy</t>
-        </is>
-      </c>
-      <c r="C687" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D687" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="E687" t="n">
-        <v>79</v>
-      </c>
-      <c r="F687" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G687" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="H687" t="n">
-        <v>51</v>
-      </c>
-      <c r="I687" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B688" t="inlineStr">
-        <is>
-          <t>Sangareddy</t>
-        </is>
-      </c>
-      <c r="C688" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D688" t="n">
-        <v>27</v>
-      </c>
-      <c r="E688" t="n">
-        <v>74</v>
-      </c>
-      <c r="F688" t="n">
-        <v>0</v>
-      </c>
-      <c r="G688" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="H688" t="n">
-        <v>3</v>
-      </c>
-      <c r="I688" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B689" t="inlineStr">
-        <is>
-          <t>Siddipet</t>
-        </is>
-      </c>
-      <c r="C689" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D689" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="E689" t="n">
-        <v>90</v>
-      </c>
-      <c r="F689" t="n">
-        <v>0</v>
-      </c>
-      <c r="G689" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H689" t="n">
-        <v>3</v>
-      </c>
-      <c r="I689" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B690" t="inlineStr">
-        <is>
-          <t>Suryapet</t>
-        </is>
-      </c>
-      <c r="C690" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D690" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="E690" t="n">
-        <v>88</v>
-      </c>
-      <c r="F690" t="n">
-        <v>0</v>
-      </c>
-      <c r="G690" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="H690" t="n">
-        <v>3</v>
-      </c>
-      <c r="I690" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B691" t="inlineStr">
-        <is>
-          <t>Vikarabad</t>
-        </is>
-      </c>
-      <c r="C691" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D691" t="n">
-        <v>26</v>
-      </c>
-      <c r="E691" t="n">
-        <v>80</v>
-      </c>
-      <c r="F691" t="n">
-        <v>0</v>
-      </c>
-      <c r="G691" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="H691" t="n">
-        <v>3</v>
-      </c>
-      <c r="I691" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="692">
-      <c r="A692" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B692" t="inlineStr">
-        <is>
-          <t>Wanaparthy</t>
-        </is>
-      </c>
-      <c r="C692" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D692" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="E692" t="n">
-        <v>73</v>
-      </c>
-      <c r="F692" t="n">
-        <v>0</v>
-      </c>
-      <c r="G692" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="H692" t="n">
-        <v>3</v>
-      </c>
-      <c r="I692" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="693">
-      <c r="A693" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B693" t="inlineStr">
-        <is>
-          <t>Warangal</t>
-        </is>
-      </c>
-      <c r="C693" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D693" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="E693" t="n">
-        <v>90</v>
-      </c>
-      <c r="F693" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G693" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="H693" t="n">
-        <v>51</v>
-      </c>
-      <c r="I693" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="694">
-      <c r="A694" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B694" t="inlineStr">
-        <is>
-          <t>Yadadri Bhuvanagiri</t>
-        </is>
-      </c>
-      <c r="C694" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="D694" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="E694" t="n">
-        <v>85</v>
-      </c>
-      <c r="F694" t="n">
-        <v>0</v>
-      </c>
-      <c r="G694" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="H694" t="n">
-        <v>3</v>
-      </c>
-      <c r="I694" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -26117,7 +24896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27408,110 +26187,49 @@
         <v>33</v>
       </c>
       <c r="D22" t="n">
-        <v>28.5</v>
+        <v>25.6</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Jogulamba Gadwal</t>
+          <t>Nalgonda</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mahabubabad</t>
+          <t>Medak</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>26.3</v>
+        <v>24.3</v>
       </c>
       <c r="I22" t="n">
-        <v>75.5</v>
+        <v>82</v>
       </c>
       <c r="J22" t="n">
-        <v>3.7</v>
+        <v>1.4</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Mancherial</t>
+          <t>Bhadradri Kothagudem</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>2.1</v>
+        <v>0.3</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Jogulamba Gadwal</t>
+          <t>Jangaon</t>
         </is>
       </c>
       <c r="N22" t="n">
-        <v>26.7</v>
+        <v>24.5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-09-24T12:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Telangana</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>33</v>
-      </c>
-      <c r="D23" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Jogulamba Gadwal</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Nizamabad</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="I23" t="n">
-        <v>85.40000000000001</v>
-      </c>
-      <c r="J23" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Bhadradri Kothagudem</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Siddipet</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>2026-09-24T18:45</t>
+          <t>2026-09-24T23:30</t>
         </is>
       </c>
     </row>
@@ -27578,7 +26296,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28.2</v>
+        <v>28.1</v>
       </c>
       <c r="D2" t="n">
         <v>31.7</v>
@@ -27587,7 +26305,7 @@
         <v>24.9</v>
       </c>
       <c r="F2" t="n">
-        <v>81.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="G2" t="n">
         <v>0.7</v>
@@ -27614,10 +26332,10 @@
         <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>82.5</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="4">
@@ -27632,7 +26350,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="D4" t="n">
         <v>33.5</v>
@@ -27641,7 +26359,7 @@
         <v>24.9</v>
       </c>
       <c r="F4" t="n">
-        <v>76</v>
+        <v>75.7</v>
       </c>
       <c r="G4" t="n">
         <v>0.8</v>
@@ -27668,10 +26386,10 @@
         <v>24.7</v>
       </c>
       <c r="F5" t="n">
-        <v>66.90000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -27686,7 +26404,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="D6" t="n">
         <v>31.4</v>
@@ -27695,10 +26413,10 @@
         <v>25.1</v>
       </c>
       <c r="F6" t="n">
-        <v>82.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -27713,7 +26431,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="D7" t="n">
         <v>32</v>
@@ -27722,10 +26440,10 @@
         <v>24.4</v>
       </c>
       <c r="F7" t="n">
-        <v>75.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
@@ -27740,7 +26458,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="D8" t="n">
         <v>33</v>
@@ -27767,7 +26485,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.9</v>
+        <v>28.7</v>
       </c>
       <c r="D9" t="n">
         <v>34.2</v>
@@ -27776,7 +26494,7 @@
         <v>23.9</v>
       </c>
       <c r="F9" t="n">
-        <v>68.40000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="G9" t="n">
         <v>4</v>
@@ -27803,7 +26521,7 @@
         <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>81</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G10" t="n">
         <v>2.3</v>
@@ -27821,7 +26539,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="D11" t="n">
         <v>32</v>
@@ -27830,10 +26548,10 @@
         <v>25.8</v>
       </c>
       <c r="F11" t="n">
-        <v>79.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
@@ -27848,16 +26566,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.5</v>
+        <v>29.6</v>
       </c>
       <c r="D12" t="n">
         <v>35.2</v>
       </c>
       <c r="E12" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="F12" t="n">
-        <v>75.5</v>
+        <v>75.2</v>
       </c>
       <c r="G12" t="n">
         <v>1.1</v>
@@ -27881,13 +26599,13 @@
         <v>32.8</v>
       </c>
       <c r="E13" t="n">
-        <v>25.2</v>
+        <v>24.8</v>
       </c>
       <c r="F13" t="n">
-        <v>82.5</v>
+        <v>82.2</v>
       </c>
       <c r="G13" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="14">
@@ -27911,10 +26629,10 @@
         <v>24.9</v>
       </c>
       <c r="F14" t="n">
-        <v>79.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="15">
@@ -27929,7 +26647,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27.3</v>
+        <v>27.1</v>
       </c>
       <c r="D15" t="n">
         <v>31.1</v>
@@ -27956,19 +26674,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28.9</v>
+        <v>28.8</v>
       </c>
       <c r="D16" t="n">
         <v>32.7</v>
       </c>
       <c r="E16" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" t="n">
-        <v>79.40000000000001</v>
+        <v>79.8</v>
       </c>
       <c r="G16" t="n">
-        <v>2.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17">
@@ -27983,7 +26701,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="D17" t="n">
         <v>30.4</v>
@@ -28019,7 +26737,7 @@
         <v>23.7</v>
       </c>
       <c r="F18" t="n">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="G18" t="n">
         <v>1.9</v>
@@ -28037,7 +26755,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.7</v>
+        <v>27.8</v>
       </c>
       <c r="D19" t="n">
         <v>32</v>
@@ -28046,7 +26764,7 @@
         <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>83.40000000000001</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="G19" t="n">
         <v>1.4</v>
@@ -28064,7 +26782,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="D20" t="n">
         <v>32.2</v>
@@ -28073,7 +26791,7 @@
         <v>23.4</v>
       </c>
       <c r="F20" t="n">
-        <v>72</v>
+        <v>72.2</v>
       </c>
       <c r="G20" t="n">
         <v>2.1</v>
@@ -28100,10 +26818,10 @@
         <v>25.7</v>
       </c>
       <c r="F21" t="n">
-        <v>67.09999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="22">
@@ -28118,7 +26836,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>27.6</v>
+        <v>27.4</v>
       </c>
       <c r="D22" t="n">
         <v>31.4</v>
@@ -28145,7 +26863,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.2</v>
+        <v>28.1</v>
       </c>
       <c r="D23" t="n">
         <v>31.6</v>
@@ -28181,7 +26899,7 @@
         <v>23.9</v>
       </c>
       <c r="F24" t="n">
-        <v>81.09999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="G24" t="n">
         <v>0.4</v>
@@ -28199,19 +26917,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="D25" t="n">
         <v>32</v>
       </c>
       <c r="E25" t="n">
-        <v>25.4</v>
+        <v>25.1</v>
       </c>
       <c r="F25" t="n">
-        <v>81.59999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="G25" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="26">
@@ -28232,7 +26950,7 @@
         <v>31.2</v>
       </c>
       <c r="E26" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="F26" t="n">
         <v>79.5</v>
@@ -28253,7 +26971,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.3</v>
+        <v>27.2</v>
       </c>
       <c r="D27" t="n">
         <v>30.8</v>
@@ -28262,10 +26980,10 @@
         <v>22.9</v>
       </c>
       <c r="F27" t="n">
-        <v>72.2</v>
+        <v>72</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="28">
@@ -28280,7 +26998,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="D28" t="n">
         <v>31.9</v>
@@ -28289,7 +27007,7 @@
         <v>23.3</v>
       </c>
       <c r="F28" t="n">
-        <v>71</v>
+        <v>70.7</v>
       </c>
       <c r="G28" t="n">
         <v>0.9</v>
@@ -28316,7 +27034,7 @@
         <v>24.2</v>
       </c>
       <c r="F29" t="n">
-        <v>80</v>
+        <v>79.8</v>
       </c>
       <c r="G29" t="n">
         <v>0.2</v>
@@ -28340,13 +27058,13 @@
         <v>34.5</v>
       </c>
       <c r="E30" t="n">
-        <v>25.4</v>
+        <v>24.8</v>
       </c>
       <c r="F30" t="n">
-        <v>71.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="G30" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="31">
@@ -28361,7 +27079,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="D31" t="n">
         <v>30.5</v>
@@ -28370,7 +27088,7 @@
         <v>22.6</v>
       </c>
       <c r="F31" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="G31" t="n">
         <v>1</v>
@@ -28388,7 +27106,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28.4</v>
+        <v>28.2</v>
       </c>
       <c r="D32" t="n">
         <v>32.1</v>
@@ -28397,7 +27115,7 @@
         <v>23.9</v>
       </c>
       <c r="F32" t="n">
-        <v>70</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G32" t="n">
         <v>3.3</v>
@@ -28415,7 +27133,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>28.9</v>
+        <v>29</v>
       </c>
       <c r="D33" t="n">
         <v>34.4</v>
@@ -28424,7 +27142,7 @@
         <v>24.7</v>
       </c>
       <c r="F33" t="n">
-        <v>74.2</v>
+        <v>73.7</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -28451,7 +27169,7 @@
         <v>24.5</v>
       </c>
       <c r="F34" t="n">
-        <v>74.2</v>
+        <v>73.8</v>
       </c>
       <c r="G34" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Update weather dataset, SQL DB, and visualization archives
</commit_message>
<xml_diff>
--- a/data/weather_data.xlsx
+++ b/data/weather_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I661"/>
+  <dimension ref="A1:I760"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24882,6 +24882,3669 @@
       <c r="I661" t="inlineStr">
         <is>
           <t>2026-09-24T23:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="E662" t="n">
+        <v>66</v>
+      </c>
+      <c r="F662" t="n">
+        <v>0</v>
+      </c>
+      <c r="G662" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="H662" t="n">
+        <v>1</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="E663" t="n">
+        <v>70</v>
+      </c>
+      <c r="F663" t="n">
+        <v>0</v>
+      </c>
+      <c r="G663" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H663" t="n">
+        <v>3</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="E664" t="n">
+        <v>65</v>
+      </c>
+      <c r="F664" t="n">
+        <v>0</v>
+      </c>
+      <c r="G664" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H664" t="n">
+        <v>3</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E665" t="n">
+        <v>68</v>
+      </c>
+      <c r="F665" t="n">
+        <v>0</v>
+      </c>
+      <c r="G665" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H665" t="n">
+        <v>3</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E666" t="n">
+        <v>66</v>
+      </c>
+      <c r="F666" t="n">
+        <v>0</v>
+      </c>
+      <c r="G666" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="H666" t="n">
+        <v>3</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E667" t="n">
+        <v>67</v>
+      </c>
+      <c r="F667" t="n">
+        <v>0</v>
+      </c>
+      <c r="G667" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H667" t="n">
+        <v>3</v>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E668" t="n">
+        <v>70</v>
+      </c>
+      <c r="F668" t="n">
+        <v>0</v>
+      </c>
+      <c r="G668" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H668" t="n">
+        <v>3</v>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="E669" t="n">
+        <v>63</v>
+      </c>
+      <c r="F669" t="n">
+        <v>0</v>
+      </c>
+      <c r="G669" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H669" t="n">
+        <v>3</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="E670" t="n">
+        <v>69</v>
+      </c>
+      <c r="F670" t="n">
+        <v>0</v>
+      </c>
+      <c r="G670" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="H670" t="n">
+        <v>3</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E671" t="n">
+        <v>66</v>
+      </c>
+      <c r="F671" t="n">
+        <v>0</v>
+      </c>
+      <c r="G671" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H671" t="n">
+        <v>3</v>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E672" t="n">
+        <v>65</v>
+      </c>
+      <c r="F672" t="n">
+        <v>0</v>
+      </c>
+      <c r="G672" t="n">
+        <v>15</v>
+      </c>
+      <c r="H672" t="n">
+        <v>3</v>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D673" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="E673" t="n">
+        <v>67</v>
+      </c>
+      <c r="F673" t="n">
+        <v>0</v>
+      </c>
+      <c r="G673" t="n">
+        <v>15</v>
+      </c>
+      <c r="H673" t="n">
+        <v>2</v>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D674" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="E674" t="n">
+        <v>65</v>
+      </c>
+      <c r="F674" t="n">
+        <v>0</v>
+      </c>
+      <c r="G674" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H674" t="n">
+        <v>3</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="E675" t="n">
+        <v>62</v>
+      </c>
+      <c r="F675" t="n">
+        <v>0</v>
+      </c>
+      <c r="G675" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H675" t="n">
+        <v>3</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="E676" t="n">
+        <v>71</v>
+      </c>
+      <c r="F676" t="n">
+        <v>0</v>
+      </c>
+      <c r="G676" t="n">
+        <v>11</v>
+      </c>
+      <c r="H676" t="n">
+        <v>3</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="E677" t="n">
+        <v>62</v>
+      </c>
+      <c r="F677" t="n">
+        <v>0</v>
+      </c>
+      <c r="G677" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H677" t="n">
+        <v>3</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E678" t="n">
+        <v>65</v>
+      </c>
+      <c r="F678" t="n">
+        <v>0</v>
+      </c>
+      <c r="G678" t="n">
+        <v>16</v>
+      </c>
+      <c r="H678" t="n">
+        <v>3</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E679" t="n">
+        <v>67</v>
+      </c>
+      <c r="F679" t="n">
+        <v>0</v>
+      </c>
+      <c r="G679" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H679" t="n">
+        <v>3</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E680" t="n">
+        <v>62</v>
+      </c>
+      <c r="F680" t="n">
+        <v>0</v>
+      </c>
+      <c r="G680" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H680" t="n">
+        <v>3</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="E681" t="n">
+        <v>61</v>
+      </c>
+      <c r="F681" t="n">
+        <v>0</v>
+      </c>
+      <c r="G681" t="n">
+        <v>15</v>
+      </c>
+      <c r="H681" t="n">
+        <v>3</v>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="E682" t="n">
+        <v>59</v>
+      </c>
+      <c r="F682" t="n">
+        <v>0</v>
+      </c>
+      <c r="G682" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H682" t="n">
+        <v>3</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D683" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E683" t="n">
+        <v>65</v>
+      </c>
+      <c r="F683" t="n">
+        <v>0</v>
+      </c>
+      <c r="G683" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H683" t="n">
+        <v>3</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="E684" t="n">
+        <v>66</v>
+      </c>
+      <c r="F684" t="n">
+        <v>0</v>
+      </c>
+      <c r="G684" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="H684" t="n">
+        <v>3</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E685" t="n">
+        <v>66</v>
+      </c>
+      <c r="F685" t="n">
+        <v>0</v>
+      </c>
+      <c r="G685" t="n">
+        <v>14</v>
+      </c>
+      <c r="H685" t="n">
+        <v>3</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E686" t="n">
+        <v>64</v>
+      </c>
+      <c r="F686" t="n">
+        <v>0</v>
+      </c>
+      <c r="G686" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="H686" t="n">
+        <v>3</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>26</v>
+      </c>
+      <c r="E687" t="n">
+        <v>64</v>
+      </c>
+      <c r="F687" t="n">
+        <v>0</v>
+      </c>
+      <c r="G687" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H687" t="n">
+        <v>3</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="E688" t="n">
+        <v>63</v>
+      </c>
+      <c r="F688" t="n">
+        <v>0</v>
+      </c>
+      <c r="G688" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="H688" t="n">
+        <v>3</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E689" t="n">
+        <v>67</v>
+      </c>
+      <c r="F689" t="n">
+        <v>0</v>
+      </c>
+      <c r="G689" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="H689" t="n">
+        <v>3</v>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E690" t="n">
+        <v>63</v>
+      </c>
+      <c r="F690" t="n">
+        <v>0</v>
+      </c>
+      <c r="G690" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H690" t="n">
+        <v>3</v>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>25</v>
+      </c>
+      <c r="E691" t="n">
+        <v>68</v>
+      </c>
+      <c r="F691" t="n">
+        <v>0</v>
+      </c>
+      <c r="G691" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H691" t="n">
+        <v>3</v>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E692" t="n">
+        <v>64</v>
+      </c>
+      <c r="F692" t="n">
+        <v>0</v>
+      </c>
+      <c r="G692" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H692" t="n">
+        <v>3</v>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E693" t="n">
+        <v>65</v>
+      </c>
+      <c r="F693" t="n">
+        <v>0</v>
+      </c>
+      <c r="G693" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H693" t="n">
+        <v>3</v>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="E694" t="n">
+        <v>59</v>
+      </c>
+      <c r="F694" t="n">
+        <v>0</v>
+      </c>
+      <c r="G694" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="H694" t="n">
+        <v>3</v>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="E695" t="n">
+        <v>62</v>
+      </c>
+      <c r="F695" t="n">
+        <v>0</v>
+      </c>
+      <c r="G695" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="H695" t="n">
+        <v>1</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E696" t="n">
+        <v>60</v>
+      </c>
+      <c r="F696" t="n">
+        <v>0</v>
+      </c>
+      <c r="G696" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H696" t="n">
+        <v>1</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D697" t="n">
+        <v>30</v>
+      </c>
+      <c r="E697" t="n">
+        <v>61</v>
+      </c>
+      <c r="F697" t="n">
+        <v>0</v>
+      </c>
+      <c r="G697" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H697" t="n">
+        <v>3</v>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D698" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="E698" t="n">
+        <v>60</v>
+      </c>
+      <c r="F698" t="n">
+        <v>0</v>
+      </c>
+      <c r="G698" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H698" t="n">
+        <v>3</v>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D699" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="E699" t="n">
+        <v>67</v>
+      </c>
+      <c r="F699" t="n">
+        <v>0</v>
+      </c>
+      <c r="G699" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H699" t="n">
+        <v>2</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D700" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E700" t="n">
+        <v>60</v>
+      </c>
+      <c r="F700" t="n">
+        <v>0</v>
+      </c>
+      <c r="G700" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="H700" t="n">
+        <v>3</v>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D701" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E701" t="n">
+        <v>61</v>
+      </c>
+      <c r="F701" t="n">
+        <v>0</v>
+      </c>
+      <c r="G701" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="H701" t="n">
+        <v>3</v>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D702" t="n">
+        <v>31</v>
+      </c>
+      <c r="E702" t="n">
+        <v>51</v>
+      </c>
+      <c r="F702" t="n">
+        <v>0</v>
+      </c>
+      <c r="G702" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="H702" t="n">
+        <v>3</v>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D703" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="E703" t="n">
+        <v>65</v>
+      </c>
+      <c r="F703" t="n">
+        <v>0</v>
+      </c>
+      <c r="G703" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="H703" t="n">
+        <v>3</v>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E704" t="n">
+        <v>64</v>
+      </c>
+      <c r="F704" t="n">
+        <v>0</v>
+      </c>
+      <c r="G704" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H704" t="n">
+        <v>3</v>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="E705" t="n">
+        <v>58</v>
+      </c>
+      <c r="F705" t="n">
+        <v>0</v>
+      </c>
+      <c r="G705" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="H705" t="n">
+        <v>2</v>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D706" t="n">
+        <v>31</v>
+      </c>
+      <c r="E706" t="n">
+        <v>61</v>
+      </c>
+      <c r="F706" t="n">
+        <v>0</v>
+      </c>
+      <c r="G706" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H706" t="n">
+        <v>3</v>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="E707" t="n">
+        <v>61</v>
+      </c>
+      <c r="F707" t="n">
+        <v>0</v>
+      </c>
+      <c r="G707" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="H707" t="n">
+        <v>2</v>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="E708" t="n">
+        <v>59</v>
+      </c>
+      <c r="F708" t="n">
+        <v>0</v>
+      </c>
+      <c r="G708" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="H708" t="n">
+        <v>3</v>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E709" t="n">
+        <v>64</v>
+      </c>
+      <c r="F709" t="n">
+        <v>0</v>
+      </c>
+      <c r="G709" t="n">
+        <v>19</v>
+      </c>
+      <c r="H709" t="n">
+        <v>3</v>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="E710" t="n">
+        <v>66</v>
+      </c>
+      <c r="F710" t="n">
+        <v>0</v>
+      </c>
+      <c r="G710" t="n">
+        <v>19</v>
+      </c>
+      <c r="H710" t="n">
+        <v>3</v>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D711" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="E711" t="n">
+        <v>60</v>
+      </c>
+      <c r="F711" t="n">
+        <v>0</v>
+      </c>
+      <c r="G711" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H711" t="n">
+        <v>3</v>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D712" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="E712" t="n">
+        <v>65</v>
+      </c>
+      <c r="F712" t="n">
+        <v>0</v>
+      </c>
+      <c r="G712" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H712" t="n">
+        <v>3</v>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D713" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E713" t="n">
+        <v>60</v>
+      </c>
+      <c r="F713" t="n">
+        <v>0</v>
+      </c>
+      <c r="G713" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="H713" t="n">
+        <v>3</v>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D714" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E714" t="n">
+        <v>54</v>
+      </c>
+      <c r="F714" t="n">
+        <v>0</v>
+      </c>
+      <c r="G714" t="n">
+        <v>18</v>
+      </c>
+      <c r="H714" t="n">
+        <v>2</v>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D715" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="E715" t="n">
+        <v>59</v>
+      </c>
+      <c r="F715" t="n">
+        <v>0</v>
+      </c>
+      <c r="G715" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="H715" t="n">
+        <v>3</v>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D716" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E716" t="n">
+        <v>65</v>
+      </c>
+      <c r="F716" t="n">
+        <v>0</v>
+      </c>
+      <c r="G716" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="H716" t="n">
+        <v>2</v>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D717" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="E717" t="n">
+        <v>65</v>
+      </c>
+      <c r="F717" t="n">
+        <v>0</v>
+      </c>
+      <c r="G717" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H717" t="n">
+        <v>1</v>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D718" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="E718" t="n">
+        <v>67</v>
+      </c>
+      <c r="F718" t="n">
+        <v>0</v>
+      </c>
+      <c r="G718" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="H718" t="n">
+        <v>3</v>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D719" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="E719" t="n">
+        <v>61</v>
+      </c>
+      <c r="F719" t="n">
+        <v>0</v>
+      </c>
+      <c r="G719" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="H719" t="n">
+        <v>3</v>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D720" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="E720" t="n">
+        <v>60</v>
+      </c>
+      <c r="F720" t="n">
+        <v>0</v>
+      </c>
+      <c r="G720" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H720" t="n">
+        <v>3</v>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D721" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="E721" t="n">
+        <v>59</v>
+      </c>
+      <c r="F721" t="n">
+        <v>0</v>
+      </c>
+      <c r="G721" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="H721" t="n">
+        <v>3</v>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D722" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="E722" t="n">
+        <v>64</v>
+      </c>
+      <c r="F722" t="n">
+        <v>0</v>
+      </c>
+      <c r="G722" t="n">
+        <v>23</v>
+      </c>
+      <c r="H722" t="n">
+        <v>3</v>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D723" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E723" t="n">
+        <v>57</v>
+      </c>
+      <c r="F723" t="n">
+        <v>0</v>
+      </c>
+      <c r="G723" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="H723" t="n">
+        <v>3</v>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D724" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="E724" t="n">
+        <v>65</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0</v>
+      </c>
+      <c r="G724" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H724" t="n">
+        <v>3</v>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D725" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="E725" t="n">
+        <v>60</v>
+      </c>
+      <c r="F725" t="n">
+        <v>0</v>
+      </c>
+      <c r="G725" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H725" t="n">
+        <v>3</v>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D726" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E726" t="n">
+        <v>60</v>
+      </c>
+      <c r="F726" t="n">
+        <v>0</v>
+      </c>
+      <c r="G726" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H726" t="n">
+        <v>3</v>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D727" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="E727" t="n">
+        <v>58</v>
+      </c>
+      <c r="F727" t="n">
+        <v>0</v>
+      </c>
+      <c r="G727" t="n">
+        <v>22</v>
+      </c>
+      <c r="H727" t="n">
+        <v>3</v>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D728" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="E728" t="n">
+        <v>60</v>
+      </c>
+      <c r="F728" t="n">
+        <v>0</v>
+      </c>
+      <c r="G728" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H728" t="n">
+        <v>0</v>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Bhadradri Kothagudem</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D729" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="E729" t="n">
+        <v>50</v>
+      </c>
+      <c r="F729" t="n">
+        <v>0</v>
+      </c>
+      <c r="G729" t="n">
+        <v>13</v>
+      </c>
+      <c r="H729" t="n">
+        <v>1</v>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Hanumakonda</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D730" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E730" t="n">
+        <v>55</v>
+      </c>
+      <c r="F730" t="n">
+        <v>0</v>
+      </c>
+      <c r="G730" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="H730" t="n">
+        <v>0</v>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D731" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E731" t="n">
+        <v>41</v>
+      </c>
+      <c r="F731" t="n">
+        <v>0</v>
+      </c>
+      <c r="G731" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H731" t="n">
+        <v>1</v>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Jagtial</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D732" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="E732" t="n">
+        <v>62</v>
+      </c>
+      <c r="F732" t="n">
+        <v>0</v>
+      </c>
+      <c r="G732" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H732" t="n">
+        <v>0</v>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Jangaon</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D733" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E733" t="n">
+        <v>50</v>
+      </c>
+      <c r="F733" t="n">
+        <v>0</v>
+      </c>
+      <c r="G733" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H733" t="n">
+        <v>0</v>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Jayashankar Bhupalpally</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D734" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E734" t="n">
+        <v>57</v>
+      </c>
+      <c r="F734" t="n">
+        <v>0</v>
+      </c>
+      <c r="G734" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H734" t="n">
+        <v>0</v>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Jogulamba Gadwal</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D735" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="E735" t="n">
+        <v>46</v>
+      </c>
+      <c r="F735" t="n">
+        <v>0</v>
+      </c>
+      <c r="G735" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H735" t="n">
+        <v>2</v>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D736" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="E736" t="n">
+        <v>53</v>
+      </c>
+      <c r="F736" t="n">
+        <v>0</v>
+      </c>
+      <c r="G736" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H736" t="n">
+        <v>0</v>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D737" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E737" t="n">
+        <v>59</v>
+      </c>
+      <c r="F737" t="n">
+        <v>0</v>
+      </c>
+      <c r="G737" t="n">
+        <v>12</v>
+      </c>
+      <c r="H737" t="n">
+        <v>0</v>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D738" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="E738" t="n">
+        <v>48</v>
+      </c>
+      <c r="F738" t="n">
+        <v>0</v>
+      </c>
+      <c r="G738" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H738" t="n">
+        <v>2</v>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Kumuram Bheem Asifabad</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E739" t="n">
+        <v>56</v>
+      </c>
+      <c r="F739" t="n">
+        <v>0</v>
+      </c>
+      <c r="G739" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H739" t="n">
+        <v>0</v>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E740" t="n">
+        <v>54</v>
+      </c>
+      <c r="F740" t="n">
+        <v>0</v>
+      </c>
+      <c r="G740" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H740" t="n">
+        <v>1</v>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Mahbubnagar</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E741" t="n">
+        <v>49</v>
+      </c>
+      <c r="F741" t="n">
+        <v>0</v>
+      </c>
+      <c r="G741" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H741" t="n">
+        <v>2</v>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Mancherial</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="E742" t="n">
+        <v>54</v>
+      </c>
+      <c r="F742" t="n">
+        <v>0</v>
+      </c>
+      <c r="G742" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="H742" t="n">
+        <v>0</v>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Medak</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E743" t="n">
+        <v>54</v>
+      </c>
+      <c r="F743" t="n">
+        <v>0</v>
+      </c>
+      <c r="G743" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H743" t="n">
+        <v>1</v>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Medchal-Malkajgiri</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="E744" t="n">
+        <v>46</v>
+      </c>
+      <c r="F744" t="n">
+        <v>0</v>
+      </c>
+      <c r="G744" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H744" t="n">
+        <v>1</v>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Mulugu</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="E745" t="n">
+        <v>58</v>
+      </c>
+      <c r="F745" t="n">
+        <v>0</v>
+      </c>
+      <c r="G745" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H745" t="n">
+        <v>0</v>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Nagarkurnool</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D746" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="E746" t="n">
+        <v>50</v>
+      </c>
+      <c r="F746" t="n">
+        <v>0</v>
+      </c>
+      <c r="G746" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H746" t="n">
+        <v>2</v>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D747" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="E747" t="n">
+        <v>41</v>
+      </c>
+      <c r="F747" t="n">
+        <v>0</v>
+      </c>
+      <c r="G747" t="n">
+        <v>13</v>
+      </c>
+      <c r="H747" t="n">
+        <v>3</v>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Narayanpet</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D748" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E748" t="n">
+        <v>52</v>
+      </c>
+      <c r="F748" t="n">
+        <v>0</v>
+      </c>
+      <c r="G748" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H748" t="n">
+        <v>1</v>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Nirmal</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D749" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E749" t="n">
+        <v>58</v>
+      </c>
+      <c r="F749" t="n">
+        <v>0</v>
+      </c>
+      <c r="G749" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H749" t="n">
+        <v>0</v>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D750" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E750" t="n">
+        <v>60</v>
+      </c>
+      <c r="F750" t="n">
+        <v>0</v>
+      </c>
+      <c r="G750" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H750" t="n">
+        <v>0</v>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Peddapalli</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D751" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="E751" t="n">
+        <v>62</v>
+      </c>
+      <c r="F751" t="n">
+        <v>0</v>
+      </c>
+      <c r="G751" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H751" t="n">
+        <v>0</v>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Rajanna Sircilla</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D752" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="E752" t="n">
+        <v>54</v>
+      </c>
+      <c r="F752" t="n">
+        <v>0</v>
+      </c>
+      <c r="G752" t="n">
+        <v>12</v>
+      </c>
+      <c r="H752" t="n">
+        <v>0</v>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D753" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="E753" t="n">
+        <v>46</v>
+      </c>
+      <c r="F753" t="n">
+        <v>0</v>
+      </c>
+      <c r="G753" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H753" t="n">
+        <v>1</v>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Sangareddy</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D754" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E754" t="n">
+        <v>44</v>
+      </c>
+      <c r="F754" t="n">
+        <v>0</v>
+      </c>
+      <c r="G754" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H754" t="n">
+        <v>1</v>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D755" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E755" t="n">
+        <v>52</v>
+      </c>
+      <c r="F755" t="n">
+        <v>0</v>
+      </c>
+      <c r="G755" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H755" t="n">
+        <v>1</v>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Suryapet</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D756" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="E756" t="n">
+        <v>46</v>
+      </c>
+      <c r="F756" t="n">
+        <v>0</v>
+      </c>
+      <c r="G756" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="H756" t="n">
+        <v>2</v>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D757" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="E757" t="n">
+        <v>49</v>
+      </c>
+      <c r="F757" t="n">
+        <v>0</v>
+      </c>
+      <c r="G757" t="n">
+        <v>9</v>
+      </c>
+      <c r="H757" t="n">
+        <v>1</v>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Wanaparthy</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D758" t="n">
+        <v>32</v>
+      </c>
+      <c r="E758" t="n">
+        <v>52</v>
+      </c>
+      <c r="F758" t="n">
+        <v>0</v>
+      </c>
+      <c r="G758" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H758" t="n">
+        <v>1</v>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D759" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E759" t="n">
+        <v>52</v>
+      </c>
+      <c r="F759" t="n">
+        <v>0</v>
+      </c>
+      <c r="G759" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H759" t="n">
+        <v>0</v>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Yadadri Bhuvanagiri</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="D760" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E760" t="n">
+        <v>45</v>
+      </c>
+      <c r="F760" t="n">
+        <v>0</v>
+      </c>
+      <c r="G760" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="H760" t="n">
+        <v>2</v>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
         </is>
       </c>
     </row>
@@ -24896,7 +28559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26230,6 +29893,189 @@
       <c r="O22" t="inlineStr">
         <is>
           <t>2026-09-24T23:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>33</v>
+      </c>
+      <c r="D23" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>25</v>
+      </c>
+      <c r="I23" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Rangareddy</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>33</v>
+      </c>
+      <c r="D24" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Vikarabad</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="I24" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Siddipet</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>23</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>33</v>
+      </c>
+      <c r="D25" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Nalgonda</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Kamareddy</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>52</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Adilabad</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Mahabubabad</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-09-27T14:00</t>
         </is>
       </c>
     </row>
@@ -26296,7 +30142,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28.1</v>
+        <v>28.3</v>
       </c>
       <c r="D2" t="n">
         <v>31.7</v>
@@ -26305,7 +30151,7 @@
         <v>24.9</v>
       </c>
       <c r="F2" t="n">
-        <v>81.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="G2" t="n">
         <v>0.7</v>
@@ -26323,7 +30169,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.5</v>
+        <v>28.7</v>
       </c>
       <c r="D3" t="n">
         <v>34.1</v>
@@ -26332,7 +30178,7 @@
         <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>82.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="G3" t="n">
         <v>2.6</v>
@@ -26350,7 +30196,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
       <c r="D4" t="n">
         <v>33.5</v>
@@ -26359,7 +30205,7 @@
         <v>24.9</v>
       </c>
       <c r="F4" t="n">
-        <v>75.7</v>
+        <v>73.7</v>
       </c>
       <c r="G4" t="n">
         <v>0.8</v>
@@ -26377,7 +30223,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="D5" t="n">
         <v>32.2</v>
@@ -26386,7 +30232,7 @@
         <v>24.7</v>
       </c>
       <c r="F5" t="n">
-        <v>66.59999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="G5" t="n">
         <v>0.9</v>
@@ -26404,7 +30250,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28</v>
+        <v>28.2</v>
       </c>
       <c r="D6" t="n">
         <v>31.4</v>
@@ -26413,7 +30259,7 @@
         <v>25.1</v>
       </c>
       <c r="F6" t="n">
-        <v>82.40000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="G6" t="n">
         <v>0.2</v>
@@ -26431,7 +30277,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.2</v>
+        <v>28.3</v>
       </c>
       <c r="D7" t="n">
         <v>32</v>
@@ -26440,7 +30286,7 @@
         <v>24.4</v>
       </c>
       <c r="F7" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G7" t="n">
         <v>0.3</v>
@@ -26458,7 +30304,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>28</v>
+        <v>28.2</v>
       </c>
       <c r="D8" t="n">
         <v>33</v>
@@ -26467,7 +30313,7 @@
         <v>24.4</v>
       </c>
       <c r="F8" t="n">
-        <v>83</v>
+        <v>80.3</v>
       </c>
       <c r="G8" t="n">
         <v>1.6</v>
@@ -26485,7 +30331,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.7</v>
+        <v>28.9</v>
       </c>
       <c r="D9" t="n">
         <v>34.2</v>
@@ -26494,7 +30340,7 @@
         <v>23.9</v>
       </c>
       <c r="F9" t="n">
-        <v>69.3</v>
+        <v>67.2</v>
       </c>
       <c r="G9" t="n">
         <v>4</v>
@@ -26512,7 +30358,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.7</v>
+        <v>26.8</v>
       </c>
       <c r="D10" t="n">
         <v>30.1</v>
@@ -26521,7 +30367,7 @@
         <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>80.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="G10" t="n">
         <v>2.3</v>
@@ -26539,7 +30385,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="D11" t="n">
         <v>32</v>
@@ -26548,7 +30394,7 @@
         <v>25.8</v>
       </c>
       <c r="F11" t="n">
-        <v>79.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="G11" t="n">
         <v>0.5</v>
@@ -26566,7 +30412,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="D12" t="n">
         <v>35.2</v>
@@ -26575,7 +30421,7 @@
         <v>25.4</v>
       </c>
       <c r="F12" t="n">
-        <v>75.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G12" t="n">
         <v>1.1</v>
@@ -26593,7 +30439,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>28.4</v>
+        <v>28.6</v>
       </c>
       <c r="D13" t="n">
         <v>32.8</v>
@@ -26602,7 +30448,7 @@
         <v>24.8</v>
       </c>
       <c r="F13" t="n">
-        <v>82.2</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G13" t="n">
         <v>0.9</v>
@@ -26620,7 +30466,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>28.6</v>
+        <v>28.8</v>
       </c>
       <c r="D14" t="n">
         <v>33.3</v>
@@ -26629,7 +30475,7 @@
         <v>24.9</v>
       </c>
       <c r="F14" t="n">
-        <v>78.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="G14" t="n">
         <v>2.9</v>
@@ -26647,7 +30493,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27.1</v>
+        <v>27.3</v>
       </c>
       <c r="D15" t="n">
         <v>31.1</v>
@@ -26656,7 +30502,7 @@
         <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>73.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="G15" t="n">
         <v>1.6</v>
@@ -26674,7 +30520,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="D16" t="n">
         <v>32.7</v>
@@ -26683,7 +30529,7 @@
         <v>25</v>
       </c>
       <c r="F16" t="n">
-        <v>79.8</v>
+        <v>77.7</v>
       </c>
       <c r="G16" t="n">
         <v>0.5</v>
@@ -26701,7 +30547,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>27</v>
+        <v>27.2</v>
       </c>
       <c r="D17" t="n">
         <v>30.4</v>
@@ -26710,7 +30556,7 @@
         <v>24</v>
       </c>
       <c r="F17" t="n">
-        <v>80</v>
+        <v>77.5</v>
       </c>
       <c r="G17" t="n">
         <v>1.1</v>
@@ -26728,7 +30574,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="D18" t="n">
         <v>31.1</v>
@@ -26737,7 +30583,7 @@
         <v>23.7</v>
       </c>
       <c r="F18" t="n">
-        <v>75.5</v>
+        <v>73</v>
       </c>
       <c r="G18" t="n">
         <v>1.9</v>
@@ -26755,7 +30601,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.8</v>
+        <v>27.9</v>
       </c>
       <c r="D19" t="n">
         <v>32</v>
@@ -26764,7 +30610,7 @@
         <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>83.09999999999999</v>
+        <v>80.5</v>
       </c>
       <c r="G19" t="n">
         <v>1.4</v>
@@ -26782,7 +30628,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27.7</v>
+        <v>27.8</v>
       </c>
       <c r="D20" t="n">
         <v>32.2</v>
@@ -26791,7 +30637,7 @@
         <v>23.4</v>
       </c>
       <c r="F20" t="n">
-        <v>72.2</v>
+        <v>70.3</v>
       </c>
       <c r="G20" t="n">
         <v>2.1</v>
@@ -26809,7 +30655,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30.2</v>
+        <v>30.3</v>
       </c>
       <c r="D21" t="n">
         <v>36.2</v>
@@ -26818,7 +30664,7 @@
         <v>25.7</v>
       </c>
       <c r="F21" t="n">
-        <v>66.8</v>
+        <v>64.8</v>
       </c>
       <c r="G21" t="n">
         <v>0.7</v>
@@ -26836,16 +30682,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>27.4</v>
+        <v>27.6</v>
       </c>
       <c r="D22" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="E22" t="n">
         <v>22.5</v>
       </c>
       <c r="F22" t="n">
-        <v>72.40000000000001</v>
+        <v>70.3</v>
       </c>
       <c r="G22" t="n">
         <v>2.7</v>
@@ -26863,7 +30709,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="D23" t="n">
         <v>31.6</v>
@@ -26872,7 +30718,7 @@
         <v>24.4</v>
       </c>
       <c r="F23" t="n">
-        <v>77.8</v>
+        <v>75.8</v>
       </c>
       <c r="G23" t="n">
         <v>0.2</v>
@@ -26890,7 +30736,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>27.3</v>
+        <v>27.5</v>
       </c>
       <c r="D24" t="n">
         <v>30.6</v>
@@ -26899,7 +30745,7 @@
         <v>23.9</v>
       </c>
       <c r="F24" t="n">
-        <v>80.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G24" t="n">
         <v>0.4</v>
@@ -26917,7 +30763,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.3</v>
+        <v>28.5</v>
       </c>
       <c r="D25" t="n">
         <v>32</v>
@@ -26926,7 +30772,7 @@
         <v>25.1</v>
       </c>
       <c r="F25" t="n">
-        <v>81.8</v>
+        <v>79.7</v>
       </c>
       <c r="G25" t="n">
         <v>0.8</v>
@@ -26944,16 +30790,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>28</v>
+        <v>28.2</v>
       </c>
       <c r="D26" t="n">
-        <v>31.2</v>
+        <v>31.3</v>
       </c>
       <c r="E26" t="n">
         <v>25.1</v>
       </c>
       <c r="F26" t="n">
-        <v>79.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="G26" t="n">
         <v>0.1</v>
@@ -26971,7 +30817,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.2</v>
+        <v>27.3</v>
       </c>
       <c r="D27" t="n">
         <v>30.8</v>
@@ -26980,7 +30826,7 @@
         <v>22.9</v>
       </c>
       <c r="F27" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G27" t="n">
         <v>0.3</v>
@@ -26998,7 +30844,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28</v>
+        <v>28.1</v>
       </c>
       <c r="D28" t="n">
         <v>31.9</v>
@@ -27007,7 +30853,7 @@
         <v>23.3</v>
       </c>
       <c r="F28" t="n">
-        <v>70.7</v>
+        <v>68.7</v>
       </c>
       <c r="G28" t="n">
         <v>0.9</v>
@@ -27025,16 +30871,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="D29" t="n">
-        <v>30.2</v>
+        <v>30.4</v>
       </c>
       <c r="E29" t="n">
         <v>24.2</v>
       </c>
       <c r="F29" t="n">
-        <v>79.8</v>
+        <v>77.3</v>
       </c>
       <c r="G29" t="n">
         <v>0.2</v>
@@ -27052,7 +30898,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>29.7</v>
+        <v>29.8</v>
       </c>
       <c r="D30" t="n">
         <v>34.5</v>
@@ -27061,7 +30907,7 @@
         <v>24.8</v>
       </c>
       <c r="F30" t="n">
-        <v>70.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G30" t="n">
         <v>0.7</v>
@@ -27079,7 +30925,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="D31" t="n">
         <v>30.5</v>
@@ -27088,7 +30934,7 @@
         <v>22.6</v>
       </c>
       <c r="F31" t="n">
-        <v>72.8</v>
+        <v>71.2</v>
       </c>
       <c r="G31" t="n">
         <v>1</v>
@@ -27106,7 +30952,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28.2</v>
+        <v>28.3</v>
       </c>
       <c r="D32" t="n">
         <v>32.1</v>
@@ -27115,7 +30961,7 @@
         <v>23.9</v>
       </c>
       <c r="F32" t="n">
-        <v>70.40000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G32" t="n">
         <v>3.3</v>
@@ -27133,7 +30979,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>29</v>
+        <v>29.1</v>
       </c>
       <c r="D33" t="n">
         <v>34.4</v>
@@ -27142,7 +30988,7 @@
         <v>24.7</v>
       </c>
       <c r="F33" t="n">
-        <v>73.7</v>
+        <v>71.8</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -27160,7 +31006,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>27.9</v>
+        <v>28.1</v>
       </c>
       <c r="D34" t="n">
         <v>32</v>
@@ -27169,7 +31015,7 @@
         <v>24.5</v>
       </c>
       <c r="F34" t="n">
-        <v>73.8</v>
+        <v>71.2</v>
       </c>
       <c r="G34" t="n">
         <v>0.5</v>

</xml_diff>